<commit_message>
Update scholarship master's program sheet with newly researched rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NFQSee5b6exfTug1PTznVN
</commit_message>
<xml_diff>
--- a/全奖硕士-已补全.xlsx
+++ b/全奖硕士-已补全.xlsx
@@ -728,7 +728,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -805,13 +805,16 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1931,16 +1934,32 @@
           <t>系明文'保证为录取学生提供资助';20 hr/wk=$14,625/yr+100% 学费;10 hr=$7,325+75% 学费;医保补贴</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n"/>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>⚠️ 不需要(推断):terminal MA按项目整体录取,官网未见套磁要求;可先邮件 jmthoma4@olemiss.edu 了解方向</t>
+        </is>
+      </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
           <t>⚠️ 未明确;联系 jmthoma4@olemiss.edu</t>
         </is>
       </c>
       <c r="H15" s="4" t="n"/>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
-      <c r="K15" s="4" t="n"/>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>不需要(研究生院页面将 Sociology MA 列为不要求 GRE/GMAT 的项目,页面表述略含糊)</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>⚠️ 不明确:研究生院称所有国际生硕博申请须提交 TOEFL(最低79,2年内有效),未见美国学位豁免条款,建议邮件确认</t>
+        </is>
+      </c>
+      <c r="K15" s="23" t="inlineStr">
+        <is>
+          <t>jmthoma4@olemiss.edu(社会学研究生项目联系人);gschool@olemiss.edu(研究生院)</t>
+        </is>
+      </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
           <t>https://olemiss.edu/socanth/academics/ma-sociology/</t>
@@ -2291,7 +2310,11 @@
 所有获得助理职位录用通知的申请者面试后将收到正式录用通知书。</t>
         </is>
       </c>
-      <c r="F21" s="12" t="n"/>
+      <c r="F21" s="26" t="inlineStr">
+        <is>
+          <t>必须:需与HES内有导师的实验室联系并获得临时录取(provisional acceptance)才能被录取</t>
+        </is>
+      </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
           <t>与HES内有导师的具体实验室联系并临时录取
@@ -2311,8 +2334,16 @@
 8月31日春季入学。</t>
         </is>
       </c>
-      <c r="I21" s="12" t="n"/>
-      <c r="J21" s="12" t="n"/>
+      <c r="I21" s="26" t="inlineStr">
+        <is>
+          <t>⚠️ 系官网未提及GRE,疑似不需要,建议邮件确认</t>
+        </is>
+      </c>
+      <c r="J21" s="26" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:研究生院对近期获得美国大学学位者豁免TOEFL/IELTS);否则 TOEFL ≥80,IELTS ≥6.5</t>
+        </is>
+      </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
           <t>heather.leach@colostate.edu
@@ -2379,7 +2410,11 @@
           <t>可选的</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n"/>
+      <c r="J22" s="27" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:研究生院对5年内获美国学位者豁免);但当TA需TOEFL口语≥24(2026/1/21后新版口语≥5.0)或通过校内口语评估(EPI)</t>
+        </is>
+      </c>
       <c r="K22" s="12" t="n"/>
       <c r="L22" s="15" t="inlineStr">
         <is>
@@ -2419,15 +2454,31 @@
           <t>我们是一个以导师为驱动的项目，申请我们的研究生项目前，与潜在的导师建立联系非常重要。与导师的联系至关重要，因为他们会支持你的申请并在申请过程中为你争取权益。通常被录取的学生已经与他们希望共事的教师进行了交流并建立了一定的关系。</t>
         </is>
       </c>
-      <c r="G23" s="12" t="n"/>
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>可以申请(多数学生获TA/RA,全额助教含学费减免+津贴)。研究生院最低GPA 3.0(低于3.0不审);需500字内个人陈述、研究陈述(thesis)、3封推荐信</t>
+        </is>
+      </c>
       <c r="H23" s="14" t="inlineStr">
         <is>
           <t>硕士的秋季申请截止日期是12月1日。</t>
         </is>
       </c>
-      <c r="I23" s="12" t="n"/>
-      <c r="J23" s="12" t="n"/>
-      <c r="K23" s="12" t="n"/>
+      <c r="I23" s="27" t="inlineStr">
+        <is>
+          <t>⚠️ 系官网未见GRE要求,疑似不需要,建议邮件确认</t>
+        </is>
+      </c>
+      <c r="J23" s="27" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:2年内获美国区域认证大学学士及以上学位可豁免,需申请后提交豁免表);否则 TOEFL ≥80,IELTS ≥6.5,Duolingo ≥110</t>
+        </is>
+      </c>
+      <c r="K23" s="27" t="inlineStr">
+        <is>
+          <t>hkgradprogram@utah.edu(H&amp;K研究生项目办公室,项目经理 Andrea Moss)</t>
+        </is>
+      </c>
       <c r="L23" s="15" t="inlineStr">
         <is>
           <t>https://health.utah.edu/health-kinesiology/graduate-programs/faq</t>
@@ -2460,13 +2511,29 @@
           <t>运动机能与健康部门为研究生提供多项机会（~7个） 每年为校内硕士生提供助教职位，传统两年制 程序。在线教育或快速入门项目的硕士生通常都是 未被考虑申请研究生助理职位。大多数助教项目覆盖所有学费 以及学年内支付学费和津贴 （9月至5月）。如需申请研究生助理职位，请填写 K&amp;H补充申请表，一旦你开始申请，将会发送给你 怀俄明大学申请。</t>
         </is>
       </c>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="26" t="n">
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>必须:须先找到研究生导师,建议9月至次年1月联系潜在导师,否则不太可能被录取或获GA推荐</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>可以申请(校内两年制硕士每年约7个TA名额,需填K&amp;H补充申请表)。本科最好为健康/运动科学/运动机能学/体育;其他专业可临时录取并补修人体解剖、人体系统生理学、运动生理学等;GPA≥3.0,3封推荐信</t>
+        </is>
+      </c>
+      <c r="H24" s="28" t="n">
         <v>46054</v>
       </c>
-      <c r="I24" s="12" t="n"/>
-      <c r="J24" s="12" t="n"/>
+      <c r="I24" s="27" t="inlineStr">
+        <is>
+          <t>可选(不要求,可提交以增强申请)</t>
+        </is>
+      </c>
+      <c r="J24" s="27" t="inlineStr">
+        <is>
+          <t>⚠️ 不明确:非英语母语者需 TOEFL ≥76(iBT)/IELTS ≥6.5;研究生院未明示美国学位豁免(各系页面说法不一),建议邮件确认;当TA另需通过 OPIc 口语考试(可由导师申请豁免)</t>
+        </is>
+      </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
           <t>Division of Kinesiology and Health
@@ -2508,16 +2575,36 @@
           <t>merit 50–100%学费+REAL带薪工作+APE award;优先截止前自动考虑</t>
         </is>
       </c>
-      <c r="F25" s="18" t="n"/>
-      <c r="G25" s="19" t="inlineStr">
-        <is>
-          <t>可</t>
-        </is>
-      </c>
-      <c r="H25" s="18" t="n"/>
-      <c r="I25" s="18" t="n"/>
-      <c r="J25" s="18" t="n"/>
-      <c r="K25" s="18" t="n"/>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取(SOPHAS申请),个人陈述可写感兴趣方向</t>
+        </is>
+      </c>
+      <c r="G25" s="29" t="inlineStr">
+        <is>
+          <t>可以申请(优先截止前完成申请自动考虑merit奖学金)。MPH无特定本科专业要求;Biostatistics等方向可能有数学先修,建议查看具体系要求</t>
+        </is>
+      </c>
+      <c r="H25" s="29" t="inlineStr">
+        <is>
+          <t>奖学金优先 2027/1/5;国际生建议 2027/5/1 前;最终 2027/7/15</t>
+        </is>
+      </c>
+      <c r="I25" s="29" t="inlineStr">
+        <is>
+          <t>不需要(多数项目不考虑GRE;Biostatistics 方向为可选)</t>
+        </is>
+      </c>
+      <c r="J25" s="29" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:在美国院校完成学位可豁免);否则 TOEFL iBT ≥79-80,IELTS ≥6</t>
+        </is>
+      </c>
+      <c r="K25" s="29" t="inlineStr">
+        <is>
+          <t>sphadmissions@emory.edu(Rollins 招生办公室,404-727-3956)</t>
+        </is>
+      </c>
       <c r="L25" s="20" t="inlineStr">
         <is>
           <t>https://sph.emory.edu/admissions/tuition-funding/scholarships</t>
@@ -2666,32 +2753,32 @@
           <t>25% GRA 为主:月薪+学费+医保;~70% MHA 生获系资助</t>
         </is>
       </c>
-      <c r="F28" s="28" t="inlineStr">
+      <c r="F28" s="26" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取(每年20–25人),滚动审核,有线上/线下面试</t>
         </is>
       </c>
-      <c r="G28" s="28" t="inlineStr">
+      <c r="G28" s="26" t="inlineStr">
         <is>
           <t>可以申请(⚠️ 原备注:国际生能否获资助未明确)。先修:各专业均可,无指定先修课;最低GPA 3.0;3封推荐信(建议≥1学术+≥1职业);医疗相关经历非必需但加分</t>
         </is>
       </c>
-      <c r="H28" s="28" t="inlineStr">
+      <c r="H28" s="26" t="inlineStr">
         <is>
           <t>奖学金/助研优先 2026/12/1;最终 2027/3/1(⚠️ 另一官网页写5/1,之后视名额滚动)(按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I28" s="28" t="inlineStr">
+      <c r="I28" s="26" t="inlineStr">
         <is>
           <t>不需要</t>
         </is>
       </c>
-      <c r="J28" s="28" t="inlineStr">
+      <c r="J28" s="26" t="inlineStr">
         <is>
           <t>否(美国认证院校学位豁免);否则 TOEFL iBT 建议 ≥100</t>
         </is>
       </c>
-      <c r="K28" s="28" t="inlineStr">
+      <c r="K28" s="26" t="inlineStr">
         <is>
           <t>karen-hammar@uiowa.edu(MHA项目主任 Karen Hammar)</t>
         </is>
@@ -2728,7 +2815,7 @@
           <t>'多数 MS 生获 2 年支持';50% TA/RA + 硕士 fellowship</t>
         </is>
       </c>
-      <c r="F29" s="28" t="inlineStr">
+      <c r="F29" s="26" t="inlineStr">
         <is>
           <t>⚠️ 建议:资助为TA/RA,建议提前联系方向匹配的教师(官网未明确要求)</t>
         </is>
@@ -2738,22 +2825,22 @@
           <t>✅ 国际生可持(教学需英语)</t>
         </is>
       </c>
-      <c r="H29" s="28" t="inlineStr">
+      <c r="H29" s="26" t="inlineStr">
         <is>
           <t>2027/2/1(仅秋季入学)</t>
         </is>
       </c>
-      <c r="I29" s="28" t="inlineStr">
+      <c r="I29" s="26" t="inlineStr">
         <is>
           <t>可选(推荐但不要求)</t>
         </is>
       </c>
-      <c r="J29" s="28" t="inlineStr">
+      <c r="J29" s="26" t="inlineStr">
         <is>
           <t>是:SIU仅豁免美国硕士学位,美本不豁免;TOEFL iBT ≥80 / IELTS ≥6.5;当TA需通过ITA Interview</t>
         </is>
       </c>
-      <c r="K29" s="28" t="inlineStr">
+      <c r="K29" s="26" t="inlineStr">
         <is>
           <t>geog@siu.edu(地理系);gradschl@siu.edu(研究生院)</t>
         </is>
@@ -2790,7 +2877,7 @@
           <t>TA/RA:学费奖学金+津贴(15-20 hr);Graduate Recruitment Scholarship(5 hr)覆盖大部分学费;1-15 截止</t>
         </is>
       </c>
-      <c r="F30" s="28" t="inlineStr">
+      <c r="F30" s="26" t="inlineStr">
         <is>
           <t>⚠️ 建议:可先联系研究生主任 Dr. Tom Smucker 了解方向匹配;官网未要求套磁</t>
         </is>
@@ -2800,17 +2887,17 @@
           <t>✅ 明文'国内外申请者按 merit 同等考虑'</t>
         </is>
       </c>
-      <c r="H30" s="28" t="inlineStr">
+      <c r="H30" s="26" t="inlineStr">
         <is>
           <t>资助考虑截止 2027/1/15(⚠️ 官网为资助全面考虑日,非明确录取截止,建议1/15前提交)</t>
         </is>
       </c>
-      <c r="I30" s="28" t="inlineStr">
+      <c r="I30" s="26" t="inlineStr">
         <is>
           <t>不需要</t>
         </is>
       </c>
-      <c r="J30" s="28" t="inlineStr">
+      <c r="J30" s="26" t="inlineStr">
         <is>
           <t>⚠️ 不明确:官网要求非英语母语者提交 TOEFL/IELTS,未见美国学位豁免说明(⚠️ 第三方:TOEFL 80 / IELTS 6.5 / Duolingo 115),建议邮件确认</t>
         </is>
@@ -2848,7 +2935,7 @@
           <t>'All applicants, domestic and international, are considered for multi-year guaranteed funding packages…typically 2 years for MS';TA含stipend+医保+学费减免</t>
         </is>
       </c>
-      <c r="F31" s="28" t="inlineStr">
+      <c r="F31" s="26" t="inlineStr">
         <is>
           <t>不需要:国内外申请者统一考虑多年资助包;⚠️ 个人陈述写明方向/教授,建议提前联系潜在导师</t>
         </is>
@@ -2858,22 +2945,22 @@
           <t>可</t>
         </is>
       </c>
-      <c r="H31" s="28" t="inlineStr">
+      <c r="H31" s="26" t="inlineStr">
         <is>
           <t>2026/12/15(仅秋季入学;⚠️ 日期见于Cartography/GIS thesis页,MS Geography同期但未单独核实)</t>
         </is>
       </c>
-      <c r="I31" s="28" t="inlineStr">
+      <c r="I31" s="26" t="inlineStr">
         <is>
           <t>不接受:系里自2020秋起不要求也不考虑GRE</t>
         </is>
       </c>
-      <c r="J31" s="28" t="inlineStr">
+      <c r="J31" s="26" t="inlineStr">
         <is>
           <t>⚠️ 大概率否:要求母语非英语或本科非英语授课者提交 TOEFL/IELTS,美本英语授课通常可豁免,建议确认</t>
         </is>
       </c>
-      <c r="K31" s="28" t="inlineStr">
+      <c r="K31" s="26" t="inlineStr">
         <is>
           <t>gradschool@geography.wisc.edu(研究生项目主任/招生)</t>
         </is>
@@ -2910,7 +2997,7 @@
           <t>'strives to provide support for all students who require it'(TA/RA),MA资助2年,TA学费减免</t>
         </is>
       </c>
-      <c r="F32" s="28" t="inlineStr">
+      <c r="F32" s="26" t="inlineStr">
         <is>
           <t>强烈建议:官网称联系潜在导师是关键步骤,录取看 merit 与教师研究匹配</t>
         </is>
@@ -2920,12 +3007,12 @@
           <t>未说明</t>
         </is>
       </c>
-      <c r="H32" s="28" t="inlineStr">
+      <c r="H32" s="26" t="inlineStr">
         <is>
           <t>研究生院资助/fellowship 2026/12/12;系资助 2027/1/10(按往年周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I32" s="28" t="inlineStr">
+      <c r="I32" s="26" t="inlineStr">
         <is>
           <t>不需要(研究生院页面;⚠️ Peterson's 仍列GRE,可能过时)</t>
         </is>
@@ -2964,22 +3051,22 @@
           <t>'Our small, tightly-knit cohorts are mostly fully funded and receive stipend and tuition remission'</t>
         </is>
       </c>
-      <c r="F33" s="28" t="inlineStr">
+      <c r="F33" s="26" t="inlineStr">
         <is>
           <t>必须:最终录取需一名教师同意指导;官网强烈建议申请前联系教师,资助多来自导师科研经费(GRA)</t>
         </is>
       </c>
-      <c r="G33" s="28" t="inlineStr">
+      <c r="G33" s="26" t="inlineStr">
         <is>
           <t>可以申请(原备注:未说明)。先修:欢迎非地理专业背景;MA需外语能力,MS不需;需2–3页陈述(写明意向导师及是否已联系)、3封推荐信</t>
         </is>
       </c>
-      <c r="H33" s="28" t="inlineStr">
+      <c r="H33" s="26" t="inlineStr">
         <is>
           <t>资助优先 2027/1/15;秋季最终 2027/5/1(⚠️ Peterson's 称国际生1/15)</t>
         </is>
       </c>
-      <c r="I33" s="28" t="inlineStr">
+      <c r="I33" s="26" t="inlineStr">
         <is>
           <t>⚠️ 不需要(官网未列GRE;Peterson's 称需GRE≥297,可能过时)</t>
         </is>
@@ -3018,16 +3105,36 @@
           <t>'Assistantships include a tuition waiver and a monthly stipend';'TA for M.S. students are typically funded for two years'</t>
         </is>
       </c>
-      <c r="F34" s="12" t="n"/>
-      <c r="G34" s="12" t="inlineStr">
-        <is>
-          <t>未说明</t>
-        </is>
-      </c>
-      <c r="H34" s="12" t="n"/>
-      <c r="I34" s="12" t="n"/>
-      <c r="J34" s="12" t="n"/>
-      <c r="K34" s="12" t="n"/>
+      <c r="F34" s="26" t="inlineStr">
+        <is>
+          <t>⚠️ 建议:官网未明确要求套磁;可先联系研究生事务教师 Walker Ashley 了解导师/助教情况</t>
+        </is>
+      </c>
+      <c r="G34" s="26" t="inlineStr">
+        <is>
+          <t>可以申请(助教含学费减免+月津贴,硕士通常资助两年)。优先 Atmospheric Science/Earth Science/Geography/Geology 或相关专业,其他专业有大量相关课程也可;需2封推荐信+CV</t>
+        </is>
+      </c>
+      <c r="H34" s="26" t="inlineStr">
+        <is>
+          <t>秋季资助考虑 2027/2/1(春季 10/1);⚠️ 研究生院通用截止 秋季 8/1(国际生 5/1),以系为准</t>
+        </is>
+      </c>
+      <c r="I34" s="26" t="inlineStr">
+        <is>
+          <t>不需要</t>
+        </is>
+      </c>
+      <c r="J34" s="26" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:研究生院认可在美国认证院校获得的学士及以上学位为英语能力证明);否则 TOEFL ≥80,IELTS ≥6.5,PTE ≥53</t>
+        </is>
+      </c>
+      <c r="K34" s="26" t="inlineStr">
+        <is>
+          <t>washley@niu.edu(研究生事务/指导 Walker Ashley);askeae@niu.edu(系通用邮箱)</t>
+        </is>
+      </c>
       <c r="L34" s="12" t="inlineStr">
         <is>
           <t>https://www.niu.edu/earth-atmosphere-environment/graduate/index.shtml</t>
@@ -3060,16 +3167,36 @@
           <t>年 &gt;$40 万 merit 支持;~60% 入学生获 offer;1/4 时 GA=$5,710/学期+全额学费减免;12-15 优先</t>
         </is>
       </c>
-      <c r="F35" s="12" t="n"/>
-      <c r="G35" s="12" t="inlineStr">
-        <is>
-          <t>✅ 明文'国内外申请者自动考虑'</t>
-        </is>
-      </c>
-      <c r="H35" s="12" t="n"/>
-      <c r="I35" s="12" t="n"/>
-      <c r="J35" s="12" t="n"/>
-      <c r="K35" s="12" t="n"/>
+      <c r="F35" s="26" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取,无需提前联系导师</t>
+        </is>
+      </c>
+      <c r="G35" s="26" t="inlineStr">
+        <is>
+          <t>可以申请(明文国内外申请者自动考虑merit资助;约60%入学生获offer)。⚠️ 官网未见特定本科专业/先修课要求;需满足研究生院GPA要求(通常最后60学分≥3.0)</t>
+        </is>
+      </c>
+      <c r="H35" s="26" t="inlineStr">
+        <is>
+          <t>资助优先 2026/12/15;最终 2027/1/15(申请窗口 2026/9/15 开放;2月底出结果)</t>
+        </is>
+      </c>
+      <c r="I35" s="26" t="inlineStr">
+        <is>
+          <t>不接受(系明确不要求也不审阅GRE成绩)</t>
+        </is>
+      </c>
+      <c r="J35" s="26" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:研究生院对5年内获美国学位者豁免);当TA需TOEFL口语达标(新版≥5.0)或通过校内口语评估</t>
+        </is>
+      </c>
+      <c r="K35" s="26" t="inlineStr">
+        <is>
+          <t>agreen4@illinois.edu(Andrew Greenlee 教授,MUP申请咨询);jakowal@illinois.edu(Jennifer Kowalski)</t>
+        </is>
+      </c>
       <c r="L35" s="12" t="inlineStr">
         <is>
           <t>https://urban.illinois.edu/programs-applying/financial-aid/</t>
@@ -3102,16 +3229,36 @@
           <t>'所有 assistant 工作 20 hr/wk 换津贴+9 学分学费减免';项目主任任命;'非常成功'安置学生</t>
         </is>
       </c>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="12" t="inlineStr">
-        <is>
-          <t>⚠️ 未明确</t>
-        </is>
-      </c>
-      <c r="H36" s="12" t="n"/>
-      <c r="I36" s="12" t="n"/>
-      <c r="J36" s="12" t="n"/>
-      <c r="K36" s="12" t="n"/>
+      <c r="F36" s="26" t="inlineStr">
+        <is>
+          <t>必须:申请时需在系内选择1-2名教师作为潜在导师;建议提前联系</t>
+        </is>
+      </c>
+      <c r="G36" s="26" t="inlineStr">
+        <is>
+          <t>可以申请(助教20小时/周换津贴+学费减免)。先修:需修过部分本科心理学课程,至少1门统计和1门研究方法;需CV、个人陈述(研究兴趣)、3封推荐信</t>
+        </is>
+      </c>
+      <c r="H36" s="26" t="inlineStr">
+        <is>
+          <t>全面考虑 2027/1/10(含推荐信);最终 2027/3/1;2月下旬面试(按2026周期日期,2027待公布)</t>
+        </is>
+      </c>
+      <c r="I36" s="26" t="inlineStr">
+        <is>
+          <t>可选(Applied Research/Experimental/Quantitative 方向可选;Behavior Analysis 方向不需要)</t>
+        </is>
+      </c>
+      <c r="J36" s="26" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:研究生院目录明文美国认证院校学士及以上学位成绩单可满足英语要求);否则 TOEFL iBT ≥80(2026/1/21后新版≥4),IELTS ≥6.5</t>
+        </is>
+      </c>
+      <c r="K36" s="26" t="inlineStr">
+        <is>
+          <t>leventbc@jmu.edu(⚠️ 2026秋目录所列项目主任 Brian Leventhal,来源不一致);研究生心理学系电话 540-568-6439</t>
+        </is>
+      </c>
       <c r="L36" s="12" t="inlineStr">
         <is>
           <t>https://www.jmu.edu/chbs/gradpsyc/psycsciences/assistantships.shtml</t>
@@ -3144,16 +3291,36 @@
           <t>'系向一年级学生授予 GA':月薪+秋春夏学费减免;Berk 发展心理 fellowship(2 年级)</t>
         </is>
       </c>
-      <c r="F37" s="12" t="n"/>
-      <c r="G37" s="12" t="inlineStr">
-        <is>
-          <t>✅ 明文'符合美国移民法就业资格即可'</t>
-        </is>
-      </c>
-      <c r="H37" s="12" t="n"/>
-      <c r="I37" s="12" t="n"/>
-      <c r="J37" s="12" t="n"/>
-      <c r="K37" s="12" t="n"/>
+      <c r="F37" s="26" t="inlineStr">
+        <is>
+          <t>⚠️ 不需要(推断):官网未提及需提前联系导师,按项目整体录取;可联系发展心理方向协调员了解</t>
+        </is>
+      </c>
+      <c r="G37" s="26" t="inlineStr">
+        <is>
+          <t>可以申请(明文符合美国移民法就业资格即可获GA;TA另需TOEFL口语≥26)。先修:心理学或相关专业(如HDFS、教育心理);建议统计+研究方法合计≥6学分及1门人类发展课程</t>
+        </is>
+      </c>
+      <c r="H37" s="26" t="inlineStr">
+        <is>
+          <t>秋季 2026/12/1(仅秋季入学)</t>
+        </is>
+      </c>
+      <c r="I37" s="26" t="inlineStr">
+        <is>
+          <t>不需要(不用于评估;可提交以证明数学能力)</t>
+        </is>
+      </c>
+      <c r="J37" s="26" t="inlineStr">
+        <is>
+          <t>⚠️ 不明确:学校国际招生页仅列英语国家豁免,未见美国学位豁免明文;TOEFL iBT ≥79-81,IELTS ≥6.5;当TA需TOEFL口语≥26(州法要求,即使录取豁免也需满足)。建议邮件 InternationalAdmissions@IllinoisState.edu 确认</t>
+        </is>
+      </c>
+      <c r="K37" s="26" t="inlineStr">
+        <is>
+          <t>ljfinan@IllinoisState.edu(发展心理学研究生协调员 Laura Finan);hdeland@IllinoisState.edu(研究生项目办公室经理)</t>
+        </is>
+      </c>
       <c r="L37" s="12" t="inlineStr">
         <is>
           <t>https://psychology.illinoisstate.edu/academics/scholarships/</t>
@@ -3480,29 +3647,29 @@
           <t>'Approximately eighty percent of our master's students receive financial assistance';奖学金仅覆盖学费,无stipend</t>
         </is>
       </c>
-      <c r="F45" s="28" t="inlineStr">
+      <c r="F45" s="26" t="inlineStr">
         <is>
           <t>MEM: 不需要:按项目整体录取,陈述中可写感兴趣的教授
 MESc: 必须:研究型学位,申请前需联系导师并列出意向教师(⚠️目录称需导师出具同意信)</t>
         </is>
       </c>
-      <c r="G45" s="28" t="inlineStr">
+      <c r="G45" s="26" t="inlineStr">
         <is>
           <t>可以申请(国际生可获YSE奖学金,约80%硕士生获资助,仅抵学费)。无硬性先修课和最低GPA;强烈建议修过生态学/生态系统、自然科学、社会科学、微观经济学和统计学;MEM入学时需具备上述基础(统计可修学院提供的非学分预备课)。</t>
         </is>
       </c>
       <c r="H45" s="12" t="n"/>
-      <c r="I45" s="28" t="inlineStr">
+      <c r="I45" s="26" t="inlineStr">
         <is>
           <t>可选(GRE/GMAT/LSAT 均可选)</t>
         </is>
       </c>
-      <c r="J45" s="28" t="inlineStr">
+      <c r="J45" s="26" t="inlineStr">
         <is>
           <t>否(美国学位豁免:本科全程在英语授课院校可申请豁免);否则需 TOEFL iBT ≥100 / IELTS ≥7.0(单项≥6.5),不接受 Duolingo</t>
         </is>
       </c>
-      <c r="K45" s="28" t="inlineStr">
+      <c r="K45" s="26" t="inlineStr">
         <is>
           <t>admissions.yse@yale.edu(YSE招生与资助办公室);⚠️ quetcy.maldonado@yale.edu(硕士项目协调员,需确认是否在任)</t>
         </is>
@@ -3539,28 +3706,28 @@
           <t>'tries very hard to make sure all graduate students have financial support in the form of Graduate Assistantships';GRA/GTA享州内学费,GTA另有学费减免;GTA考虑截止3/1</t>
         </is>
       </c>
-      <c r="F46" s="28" t="inlineStr">
+      <c r="F46" s="26" t="inlineStr">
         <is>
           <t>必须:论文型MS须有教师同意担任导师才会被录取,资助多由导师的GRA经费提供</t>
         </is>
       </c>
-      <c r="G46" s="28" t="inlineStr">
+      <c r="G46" s="26" t="inlineStr">
         <is>
           <t>可以申请(⚠️ 国际生能否获GRA/GTA未见明文限制)。⚠️ 需理科相关本科背景(在线PSM明确要求);最近两年GPA≥3.0;3封推荐信(不得来自意向导师或委员会成员);个人陈述写研究兴趣与职业目标;录取前须有导师同意。</t>
         </is>
       </c>
-      <c r="H46" s="28" t="inlineStr">
+      <c r="H46" s="26" t="inlineStr">
         <is>
           <t>⚠️ LRES申请页:秋季 6/15、春季 11/1(可能针对在线Professional MS);论文型MS视导师经费录取,GTA考虑截止 3/1;建议 2027/3/1 前提交(按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I46" s="28" t="inlineStr">
+      <c r="I46" s="26" t="inlineStr">
         <is>
           <t>⚠️ 不需要:系页面未列GRE(在线PSM明确不需要),论文型建议邮件确认</t>
         </is>
       </c>
       <c r="J46" s="12" t="n"/>
-      <c r="K46" s="28" t="inlineStr">
+      <c r="K46" s="26" t="inlineStr">
         <is>
           <t>lresinfo@montana.edu(LRES系研究生项目);gradschool@montana.edu(MSU研究生院)</t>
         </is>
@@ -3597,32 +3764,32 @@
           <t>系 FAQ:'多数生统学生被任命为 TA 和/或 RA';≥25% 任命含学费奖学金+50% 费用+津贴;12-01 优先</t>
         </is>
       </c>
-      <c r="F47" s="28" t="inlineStr">
+      <c r="F47" s="26" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,TA/RA由系里统一分配;个人陈述可写感兴趣的教授</t>
         </is>
       </c>
-      <c r="G47" s="28" t="inlineStr">
+      <c r="G47" s="26" t="inlineStr">
         <is>
           <t>可以申请(国际生可获TA/RA)。需学士学位、GPA≥3.0;先修:三门微积分(单变量、积分、多元,对应MATH:1850/1860/2850)+线性代数(MATH:2700);至少会一门编程语言;建议理科/数学/健康科学背景,有统计或数据分析经验者优先。</t>
         </is>
       </c>
-      <c r="H47" s="28" t="inlineStr">
+      <c r="H47" s="26" t="inlineStr">
         <is>
           <t>资助优先 2026/12/1;最终 2027/1/10;仅秋季入学,通过SOPHAS申请(⚠️ 依据官网现行页面,2027周期请再确认)</t>
         </is>
       </c>
-      <c r="I47" s="28" t="inlineStr">
+      <c r="I47" s="26" t="inlineStr">
         <is>
           <t>不需要</t>
         </is>
       </c>
-      <c r="J47" s="28" t="inlineStr">
+      <c r="J47" s="26" t="inlineStr">
         <is>
           <t>否(美国学位豁免:美国认证大学学士自动豁免);否则 TOEFL iBT ≥100 / IELTS ≥7.0 / Duolingo ≥120;⚠️ 当TA可能需参加校内英语口语评估</t>
         </is>
       </c>
-      <c r="K47" s="28" t="inlineStr">
+      <c r="K47" s="26" t="inlineStr">
         <is>
           <t>biostatistics@uiowa.edu(生统系研究生项目管理员);admissions@uiowa.edu(UIowa招生办)</t>
         </is>
@@ -4331,7 +4498,7 @@
           <t>'Students admitted to all graduate programs in SPHHS are eligible to receive on-campus assistantships';'Each assistantship includes a stipend, tuition waiver, and health-fee waiver'</t>
         </is>
       </c>
-      <c r="F64" s="29" t="inlineStr">
+      <c r="F64" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取(SOPHAS),个人陈述可写感兴趣的HPM教授;MS偏研究,可选择性提前联系项目主任了解匹配度</t>
         </is>
@@ -4341,22 +4508,22 @@
           <t>未说明</t>
         </is>
       </c>
-      <c r="H64" s="29" t="inlineStr">
+      <c r="H64" s="30" t="inlineStr">
         <is>
           <t>SOPHAS 截止 2/1(MS/MPH/PhD;仅秋季入学,8月中开放,建议尽早),即 2027/2/1(⚠️ 第三方显示2027周期同为2/1,官网2027年份待确认)</t>
         </is>
       </c>
-      <c r="I64" s="29" t="inlineStr">
+      <c r="I64" s="30" t="inlineStr">
         <is>
           <t>不需要(SPHHS官网:所有学位及证书项目不要求GRE/GMAT;⚠️ Peterson's仍列GRE,已过时)</t>
         </is>
       </c>
-      <c r="J64" s="29" t="inlineStr">
+      <c r="J64" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不明确:研究生院对非美国公民/永居的非母语者要求成绩,另有豁免条件(旧版研究生简章及经济系页面含'在美国获得学位'豁免,大概率可豁免,需邮件 gradadm@grad.umass.edu 确认);若需提交:TOEFL ≥80(2026年1月后新制≥4),IELTS ≥6.5,Duolingo ≥115</t>
         </is>
       </c>
-      <c r="K64" s="29" t="inlineStr">
+      <c r="K64" s="30" t="inlineStr">
         <is>
           <t>sphhsgradapply@umass.edu(SPHHS 校园项目研究生招生);abartnik@umass.edu(HPM系办公室协调员)</t>
         </is>
@@ -4393,7 +4560,7 @@
           <t>TA/RA $6,413–12,827/学期+州外学费减免+50–100%州内学费;'Priority…given to doctoral students, then master's'</t>
         </is>
       </c>
-      <c r="F65" s="29" t="inlineStr">
+      <c r="F65" s="30" t="inlineStr">
         <is>
           <t>不需要:MPH按项目整体录取,无需套磁;TA/RA优先给博士生,可在录取后联系系里/教授询问岗位</t>
         </is>
@@ -4404,17 +4571,17 @@
         </is>
       </c>
       <c r="H65" s="21" t="n"/>
-      <c r="I65" s="29" t="inlineStr">
+      <c r="I65" s="30" t="inlineStr">
         <is>
           <t>不需要(官网:GRE仅PhD Epidemiology、MS/PhD Biostatistics需要;MPH已取消GRE/MCAT要求)</t>
         </is>
       </c>
-      <c r="J65" s="29" t="inlineStr">
+      <c r="J65" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免:研究生院规定在美国区域认证院校获学士/研究生学位者免交;⚠️ 信息学院页面提及学位距入学不超过2年,建议确认)。若需:TOEFL ≥79(2026/1/21后新制≥4)</t>
         </is>
       </c>
-      <c r="K65" s="29" t="inlineStr">
+      <c r="K65" s="30" t="inlineStr">
         <is>
           <t>coph-admit@arizona.edu(公共卫生学院招生办)</t>
         </is>
@@ -4451,7 +4618,7 @@
           <t>GTA:$15,000/9 个月+外州学费豁免+大部分学费减免+医保;20 hr 教活动课</t>
         </is>
       </c>
-      <c r="F66" s="29" t="inlineStr">
+      <c r="F66" s="30" t="inlineStr">
         <is>
           <t>不需要:系里整体审核(holistic review)录取;个人陈述可提感兴趣的教授/研究方向</t>
         </is>
@@ -4462,7 +4629,7 @@
         </is>
       </c>
       <c r="H66" s="21" t="n"/>
-      <c r="I66" s="29" t="inlineStr">
+      <c r="I66" s="30" t="inlineStr">
         <is>
           <t>⚠️ 官网未提及;第三方(IDP)称最后60学分GPA&lt;3.5时需GRE,建议邮件确认</t>
         </is>
@@ -4837,16 +5004,28 @@
           <t>系有多个GTA'carry a stipend and tuition reduction'(部分学费减免)</t>
         </is>
       </c>
-      <c r="F75" s="21" t="n"/>
-      <c r="G75" s="21" t="inlineStr">
-        <is>
-          <t>可</t>
+      <c r="F75" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取;如想申GTA或做生物力学实验室研究,可提前联系系里了解岗位</t>
+        </is>
+      </c>
+      <c r="G75" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(国际生可申GTA,带stipend+部分学费减免)。先修:Exercise Science方向需≥18学分运动/体育/健身相关课程;3封推荐信(≥1封来自教授);⚠️ 最低GPA各来源不一(2.7/2.75/3.0),未达标可有条件录取</t>
         </is>
       </c>
       <c r="H75" s="21" t="n"/>
       <c r="I75" s="21" t="n"/>
-      <c r="J75" s="21" t="n"/>
-      <c r="K75" s="21" t="n"/>
+      <c r="J75" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:持美国区域认证大学学位者无需提交英语成绩);否则TOEFL ≥79,IELTS ≥6.0</t>
+        </is>
+      </c>
+      <c r="K75" s="30" t="inlineStr">
+        <is>
+          <t>ksm@usd.edu(Kinesiology &amp; Sport Management 系);gradadmissions@usd.edu(研究生招生办)</t>
+        </is>
+      </c>
       <c r="L75" s="21" t="inlineStr">
         <is>
           <t>https://www.usd.edu/Academics/Graduate-Programs/Kinesiology-and-Sport-Management</t>
@@ -4879,16 +5058,28 @@
           <t>GA竞争性;'General tuition and the non-resident fees are waived for graduate assistants';≤20h/周</t>
         </is>
       </c>
-      <c r="F76" s="21" t="n"/>
-      <c r="G76" s="21" t="inlineStr">
-        <is>
-          <t>可</t>
+      <c r="F76" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取;可联系学院主任 Dr. Stephanie McCoy Smith 咨询GA岗位</t>
+        </is>
+      </c>
+      <c r="G76" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(GA免学费及外州费)。先修:运动科学或相关本科;化学或生物1门+生理学、营养学本科课;最低GPA 2.75(最后60学分);需SOP、简历、3封推荐信。⚠️ 该方向目录标注100%在线,需确认是否有校园版/能否持F-1</t>
         </is>
       </c>
       <c r="H76" s="21" t="n"/>
       <c r="I76" s="21" t="n"/>
-      <c r="J76" s="21" t="n"/>
-      <c r="K76" s="21" t="n"/>
+      <c r="J76" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:持美国认证大学学位可免);否则TOEFL ≥71,IELTS ≥6.0</t>
+        </is>
+      </c>
+      <c r="K76" s="30" t="inlineStr">
+        <is>
+          <t>stephanie.mccoy@usm.edu(学院主任/项目顾问 Dr. Stephanie Smith);电话 601-266-5358(School of Kinesiology and Nutrition)</t>
+        </is>
+      </c>
       <c r="L76" s="21" t="inlineStr">
         <is>
           <t>https://www.usm.edu/graduate-programs/kinesiology-sport-coaching-education.php</t>
@@ -4921,16 +5112,36 @@
           <t>'Most SHPK GTAs are awarded to PhD students; however, master's students are also eligible';全年接受GTA申请</t>
         </is>
       </c>
-      <c r="F77" s="21" t="n"/>
-      <c r="G77" s="21" t="inlineStr">
-        <is>
-          <t>未说明</t>
-        </is>
-      </c>
-      <c r="H77" s="21" t="n"/>
-      <c r="I77" s="21" t="n"/>
-      <c r="J77" s="21" t="n"/>
-      <c r="K77" s="21" t="n"/>
+      <c r="F77" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取;GTA多给博士,硕士可申,建议联系方向教授表达兴趣</t>
+        </is>
+      </c>
+      <c r="G77" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(硕士也可申GTA,全年接受申请)。先修:解剖与生理学、运动生理学、3学分高年级运动科学课(可入学后补修,不计学分);最后60学分GPA ≥3.0</t>
+        </is>
+      </c>
+      <c r="H77" s="30" t="inlineStr">
+        <is>
+          <t>滚动录取;优先截止 秋季 2027/3/1(春季7/1)。国际生建议提前6–8个月准备</t>
+        </is>
+      </c>
+      <c r="I77" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 必需(研究生手册写Exercise Physiology方向需提交GRE;项目页未写,可能过时,建议确认)</t>
+        </is>
+      </c>
+      <c r="J77" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 不明确:研究生院有英语豁免表,美国本科学位应可豁免,需确认;否则TOEFL ≥79,IELTS ≥6.5,Duolingo ≥100</t>
+        </is>
+      </c>
+      <c r="K77" s="30" t="inlineStr">
+        <is>
+          <t>SHPK@twu.edu(School of Health Promotion &amp; Kinesiology)</t>
+        </is>
+      </c>
       <c r="L77" s="21" t="inlineStr">
         <is>
           <t>https://twu.edu/kinesiology/graduate-programs/</t>
@@ -4963,16 +5174,32 @@
           <t>'All qualifying applicants are considered for assistantships. You do not need to apply';1/15前申请优先考虑资助</t>
         </is>
       </c>
-      <c r="F78" s="21" t="n"/>
-      <c r="G78" s="21" t="inlineStr">
-        <is>
-          <t>未说明</t>
-        </is>
-      </c>
-      <c r="H78" s="21" t="n"/>
+      <c r="F78" s="30" t="inlineStr">
+        <is>
+          <t>不需要:硕士按项目整体录取(MS/PhD衔接轨道需导师背书);可在文书中写感兴趣教授</t>
+        </is>
+      </c>
+      <c r="G78" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(合格申请人自动考虑资助,无需单独申请)。⚠️ 项目页未列具体先修/最低GPA(同系MSAT要求GPA ≥3.0),建议运动科学相关背景</t>
+        </is>
+      </c>
+      <c r="H78" s="30" t="inlineStr">
+        <is>
+          <t>资助/优先 2027/1/15;最终 2027/7/1(视名额)</t>
+        </is>
+      </c>
       <c r="I78" s="21" t="n"/>
-      <c r="J78" s="21" t="n"/>
-      <c r="K78" s="21" t="n"/>
+      <c r="J78" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免,材料齐后招生专员手动豁免);入学后所有国际生需参加UNCG英语测评</t>
+        </is>
+      </c>
+      <c r="K78" s="30" t="inlineStr">
+        <is>
+          <t>plkocher@uncg.edu(研究生项目主任 Pam Brown);clbooth@uncg.edu(研究生协调员 Carol Booth)</t>
+        </is>
+      </c>
       <c r="L78" s="21" t="inlineStr">
         <is>
           <t>https://kin.uncg.edu/graduate-degrees/faqs/</t>
@@ -5005,16 +5232,36 @@
           <t>'Associateships provide professional experience and financial support';12/1为资助截止;无MS比例</t>
         </is>
       </c>
-      <c r="F79" s="21" t="n"/>
-      <c r="G79" s="21" t="inlineStr">
-        <is>
-          <t>未说明</t>
-        </is>
-      </c>
-      <c r="H79" s="21" t="n"/>
-      <c r="I79" s="21" t="n"/>
-      <c r="J79" s="21" t="n"/>
-      <c r="K79" s="21" t="n"/>
+      <c r="F79" s="30" t="inlineStr">
+        <is>
+          <t>建议:Associateship多与教授项目/实验室挂钩,建议联系方向匹配教授(如 kackley.19@osu.edu)</t>
+        </is>
+      </c>
+      <c r="G79" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(国际生可获GTA/GRA associateship;担任GTA需通过口语测试)。先修:4年制本科学位;⚠️ 第三方称GPA ≥3.0,官网未注明具体先修课</t>
+        </is>
+      </c>
+      <c r="H79" s="30" t="inlineStr">
+        <is>
+          <t>资助截止 2026/12/1;之后滚动录取至名额满(申请9/1开放)</t>
+        </is>
+      </c>
+      <c r="I79" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 不需要(研究生院不要求,项目页未提及),建议确认</t>
+        </is>
+      </c>
+      <c r="J79" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:须在入学前24个月内获美国学士学位);入学后需英语写作测评;当GTA需口语能力认证(OPA)</t>
+        </is>
+      </c>
+      <c r="K79" s="30" t="inlineStr">
+        <is>
+          <t>kinesiology@osu.edu(Kinesiology 研究生项目)</t>
+        </is>
+      </c>
       <c r="L79" s="21" t="inlineStr">
         <is>
           <t>https://ehe.osu.edu/graduate/kinesiology/health-and-exercise-science/ms-kinesiology</t>
@@ -5047,15 +5294,31 @@
           <t>校级GA:30学分学费减免/年+非居民学费全免+系定stipend;岗位在Workday发布</t>
         </is>
       </c>
-      <c r="F80" s="21" t="n"/>
-      <c r="G80" s="21" t="inlineStr">
-        <is>
-          <t>可</t>
-        </is>
-      </c>
-      <c r="H80" s="21" t="n"/>
-      <c r="I80" s="21" t="n"/>
-      <c r="J80" s="21" t="n"/>
+      <c r="F80" s="30" t="inlineStr">
+        <is>
+          <t>强烈建议:研究型论文硕士,依托Human Performance Lab,建议先联系研究生项目主任 Scott Trappe 或方向导师</t>
+        </is>
+      </c>
+      <c r="G80" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(GA含学费减免+非居民费全免+stipend)。先修:必须修过有机化学I+II(含实验);GPA&lt;2.75可凭其他成就有条件考虑;需CV、3封推荐信、补充表+写作样本</t>
+        </is>
+      </c>
+      <c r="H80" s="30" t="inlineStr">
+        <is>
+          <t>秋季 2027/2/1(⚠️ Peterson's 称1/15);国际生截止以研究生招生办为准</t>
+        </is>
+      </c>
+      <c r="I80" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 可能必需:第三方(Mastersportal/Peterson's)列为必需,官网页未提及,建议确认</t>
+        </is>
+      </c>
+      <c r="J80" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免:美国认证大学学位或≥24学分美国学习可免);否则TOEFL ≥79,IELTS ≥6.5;成绩2年有效</t>
+        </is>
+      </c>
       <c r="K80" s="21" t="n"/>
       <c r="L80" s="21" t="inlineStr">
         <is>
@@ -5089,16 +5352,36 @@
           <t>硕士GA stipend $10,000–12,500/年+fee remission;'Master student assistantships are for only one year'</t>
         </is>
       </c>
-      <c r="F81" s="21" t="n"/>
-      <c r="G81" s="21" t="inlineStr">
-        <is>
-          <t>可(AI需过TEPAIC)</t>
-        </is>
-      </c>
-      <c r="H81" s="21" t="n"/>
-      <c r="I81" s="21" t="n"/>
-      <c r="J81" s="21" t="n"/>
-      <c r="K81" s="21" t="n"/>
+      <c r="F81" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取</t>
+        </is>
+      </c>
+      <c r="G81" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(国际生可获GA;担任AI需通过TEPAIC口语测试)。先修:学士学位,无统一必修课(各方向可能另有要求);SOP ≤600字;经SOPHAS申请+IU研究生院补充申请</t>
+        </is>
+      </c>
+      <c r="H81" s="30" t="inlineStr">
+        <is>
+          <t>优先 2027/1/15;最终 2027/4/1(按SOPHAS中具体项目为准)</t>
+        </is>
+      </c>
+      <c r="I81" s="30" t="inlineStr">
+        <is>
+          <t>可选(SPH-B所有研究生项目GRE可选)</t>
+        </is>
+      </c>
+      <c r="J81" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免);⚠️ 部分资助机会仍可能要求英语成绩;担任AI需TEPAIC</t>
+        </is>
+      </c>
+      <c r="K81" s="30" t="inlineStr">
+        <is>
+          <t>sphgrad@iu.edu(SPH-Bloomington研究生招生)</t>
+        </is>
+      </c>
       <c r="L81" s="21" t="inlineStr">
         <is>
           <t>https://bulletins.iu.edu/iub/phb/2020-2021/graduate/financial-aid.shtml</t>
@@ -5131,16 +5414,36 @@
           <t>'Each applicant is evaluated for an assistantship. No separate application';按学期任命、无续聘保证</t>
         </is>
       </c>
-      <c r="F82" s="21" t="n"/>
-      <c r="G82" s="21" t="inlineStr">
-        <is>
-          <t>未说明</t>
-        </is>
-      </c>
-      <c r="H82" s="21" t="n"/>
-      <c r="I82" s="21" t="n"/>
-      <c r="J82" s="21" t="n"/>
-      <c r="K82" s="21" t="n"/>
+      <c r="F82" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取,所有申请人自动评估assistantship</t>
+        </is>
+      </c>
+      <c r="G82" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(国际生担任TA需通过SPEAK或TOEFL口语≥26)。无专业/先修要求,所有专业可申;本科高年级GPA ≥3.0;2封推荐信;申请费$30</t>
+        </is>
+      </c>
+      <c r="H82" s="30" t="inlineStr">
+        <is>
+          <t>资助优先 2027/2/1;早申(建议国际生)2027/4/1;最终 2027/7/1(⚠️ 国际生页另写秋季1/15,冲突,建议确认)</t>
+        </is>
+      </c>
+      <c r="I82" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 可能不需要:研究生院已对多数硕士豁免GRE(Spring 2026起无全校要求),但MPH目录仍提及GRE 50%分位,建议确认</t>
+        </is>
+      </c>
+      <c r="J82" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学士学位可豁免校级英语要求,但系可另有要求);当TA需SPEAK或TOEFL口语≥26</t>
+        </is>
+      </c>
+      <c r="K82" s="30" t="inlineStr">
+        <is>
+          <t>cosspp-publichealthinfo@fsu.edu(MPH招生);hmahony@fsu.edu(MPH项目主任 Helen Mahony)</t>
+        </is>
+      </c>
       <c r="L82" s="21" t="inlineStr">
         <is>
           <t>https://cosspp.fsu.edu/publichealth/funding-and-scholarships/</t>
@@ -5173,16 +5476,36 @@
           <t>约30%(MPH)/40%(SM)获school grants,多覆盖1/4–1/2学费;Presidential Scholars约10人全额学费</t>
         </is>
       </c>
-      <c r="F83" s="21" t="n"/>
-      <c r="G83" s="21" t="inlineStr">
-        <is>
-          <t>可</t>
-        </is>
-      </c>
-      <c r="H83" s="21" t="n"/>
-      <c r="I83" s="21" t="n"/>
-      <c r="J83" s="21" t="n"/>
-      <c r="K83" s="21" t="n"/>
+      <c r="F83" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取</t>
+        </is>
+      </c>
+      <c r="G83" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(国际生可获school grants)。MPH-65学分版需学士学位+≥2年连续全职公卫相关工作经验;SM需展示定量能力(⚠️ 各SM方向先修不同,见项目页)</t>
+        </is>
+      </c>
+      <c r="H83" s="30" t="inlineStr">
+        <is>
+          <t>2026/12/1(SOPHAS,多数项目);决定2–3月邮件通知</t>
+        </is>
+      </c>
+      <c r="I83" s="30" t="inlineStr">
+        <is>
+          <t>可选(MPH全部方向、SM-HPM为test-optional;⚠️ 其他SM方向需查项目页)</t>
+        </is>
+      </c>
+      <c r="J83" s="30" t="inlineStr">
+        <is>
+          <t>否(获得英语授课院校学位者免考)</t>
+        </is>
+      </c>
+      <c r="K83" s="30" t="inlineStr">
+        <is>
+          <t>admissions@hsph.harvard.edu(Harvard Chan 招生办)</t>
+        </is>
+      </c>
       <c r="L83" s="21" t="inlineStr">
         <is>
           <t>https://hsph.harvard.edu/tuition-and-financial-aid/types-of-financial-aid/</t>
@@ -5215,28 +5538,28 @@
           <t>'All students admitted…reviewed for institutional academic merit scholarships';$7,500–30,000/年</t>
         </is>
       </c>
-      <c r="F84" s="29" t="inlineStr">
+      <c r="F84" s="30" t="inlineStr">
         <is>
           <t>不需要:MPH/MS 经 SOPHAS 按项目整体录取,个人陈述可写感兴趣的教授/研究方向</t>
         </is>
       </c>
-      <c r="G84" s="29" t="inlineStr">
+      <c r="G84" s="30" t="inlineStr">
         <is>
           <t>可以申请(国际生仅可获 merit 奖学金;need-based 资助限美籍)。先修:MPH 接受任何本科专业,无硬性先修课;MS(如生物统计)需微积分等数理基础;⚠️ 官网未列最低 GPA</t>
         </is>
       </c>
-      <c r="H84" s="29" t="inlineStr">
+      <c r="H84" s="30" t="inlineStr">
         <is>
           <t>优先(含奖学金考虑)2026/12/1;MPH 一般截止约 2027/1/15(2026 周期曾延至 2 月)(按2026周期,2027待公布);⚠️ 第三方显示 Accelerated MPH 2027/1/15</t>
         </is>
       </c>
-      <c r="I84" s="29" t="inlineStr">
+      <c r="I84" s="30" t="inlineStr">
         <is>
           <t>可选:2026 秋季起所有硕士项目标化成绩均为可选</t>
         </is>
       </c>
       <c r="J84" s="21" t="n"/>
-      <c r="K84" s="29" t="inlineStr">
+      <c r="K84" s="30" t="inlineStr">
         <is>
           <t>ph-admit@columbia.edu(Mailman 招生办)</t>
         </is>
@@ -5273,28 +5596,28 @@
           <t>'$34M in scholarships and tuition assistance';GSI/GSRA可申;无比例</t>
         </is>
       </c>
-      <c r="F85" s="29" t="inlineStr">
+      <c r="F85" s="30" t="inlineStr">
         <is>
           <t>不需要:按系整体录取(SOPHAS),个人陈述可写感兴趣的教授;GSRA 多需录取后自行联系教授</t>
         </is>
       </c>
-      <c r="G85" s="29" t="inlineStr">
+      <c r="G85" s="30" t="inlineStr">
         <is>
           <t>可以申请(国际生可申 GSI/GSRA 及系奖学金)。先修:一般接受任何专业;Biostatistics 需微积分/线代,EHS 等需理科基础(⚠️ 按系不同);⚠️ 官网未列最低 GPA</t>
         </is>
       </c>
-      <c r="H85" s="29" t="inlineStr">
+      <c r="H85" s="30" t="inlineStr">
         <is>
           <t>资助/奖学金优先 2026/12/1;国际生最终 2027/1/15;美籍最终 2027/5/15(按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I85" s="29" t="inlineStr">
+      <c r="I85" s="30" t="inlineStr">
         <is>
           <t>⚠️ 多数项目不需要/可选(第三方 Peterson's 仍列 GRE,官网未核实,建议按具体系确认)</t>
         </is>
       </c>
       <c r="J85" s="21" t="n"/>
-      <c r="K85" s="29" t="inlineStr">
+      <c r="K85" s="30" t="inlineStr">
         <is>
           <t>⚠️ sph.inquiries@umich.edu(SPH 招生办,未经本次检索核实)</t>
         </is>
@@ -5331,16 +5654,36 @@
           <t>GTA/GRA:学费减免+医保+津贴;CHS 硕士 $1,900/月(0.5 FTE);外州学费全免</t>
         </is>
       </c>
-      <c r="F86" s="21" t="n"/>
-      <c r="G86" s="21" t="inlineStr">
-        <is>
-          <t>⚠️ 未明确</t>
-        </is>
-      </c>
-      <c r="H86" s="21" t="n"/>
-      <c r="I86" s="21" t="n"/>
-      <c r="J86" s="21" t="n"/>
-      <c r="K86" s="21" t="n"/>
+      <c r="F86" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取;GTA/GRA可联系项目协调员咨询</t>
+        </is>
+      </c>
+      <c r="G86" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(国际生可获GTA/GRA,外州学费全免)。先修:本科GPA ≥3.0;需简历/CV、2封推荐信;⚠️ 未列具体先修课</t>
+        </is>
+      </c>
+      <c r="H86" s="30" t="inlineStr">
+        <is>
+          <t>滚动录取,建议开学前≥6周提交;⚠️ 为争取GTA/GRA建议2027/3前提交</t>
+        </is>
+      </c>
+      <c r="I86" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 项目页未列要求,应为不需要,建议确认</t>
+        </is>
+      </c>
+      <c r="J86" s="30" t="inlineStr">
+        <is>
+          <t>否(英语国家英语授课学位豁免,美国学位适用);否则TOEFL ≥79,IELTS ≥6.5</t>
+        </is>
+      </c>
+      <c r="K86" s="30" t="inlineStr">
+        <is>
+          <t>darcy.mcmaughan@okstate.edu(项目协调员 Dr. DJ McMaughan)</t>
+        </is>
+      </c>
       <c r="L86" s="21" t="inlineStr">
         <is>
           <t>https://go.okstate.edu/graduate-academics/programs/masters/health-promotion-ms.html</t>
@@ -5667,28 +6010,28 @@
           <t>所有 MPH 申请者自动考虑系学费奖学金(12-01 优先);GSI/GSRA 含学费+津贴+医保</t>
         </is>
       </c>
-      <c r="F94" s="29" t="inlineStr">
+      <c r="F94" s="30" t="inlineStr">
         <is>
           <t>不需要:按系整体录取(SOPHAS),个人陈述可写感兴趣的教授;GSRA 多需录取后自行联系教授</t>
         </is>
       </c>
-      <c r="G94" s="29" t="inlineStr">
+      <c r="G94" s="30" t="inlineStr">
         <is>
           <t>可以申请(✅ 官网明文国内外申请者同等考虑系学费奖学金)。先修:一般接受任何专业;部分系(Biostat 等)需数理先修;⚠️ 未列最低 GPA</t>
         </is>
       </c>
-      <c r="H94" s="29" t="inlineStr">
+      <c r="H94" s="30" t="inlineStr">
         <is>
           <t>资助/奖学金优先 2026/12/1;国际生最终 2027/1/15;美籍最终 2027/5/15(按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I94" s="29" t="inlineStr">
+      <c r="I94" s="30" t="inlineStr">
         <is>
           <t>⚠️ 多数项目不需要/可选(第三方 Peterson's 仍列 GRE,官网未核实,建议按具体系确认)</t>
         </is>
       </c>
       <c r="J94" s="21" t="n"/>
-      <c r="K94" s="29" t="inlineStr">
+      <c r="K94" s="30" t="inlineStr">
         <is>
           <t>⚠️ sph.inquiries@umich.edu(SPH 招生办,未经本次检索核实)</t>
         </is>
@@ -6061,7 +6404,7 @@
           <t>各校有限 GRA/部分奖学金;NW 最高 $20,000 奖学金无 assistantship</t>
         </is>
       </c>
-      <c r="F103" s="29" t="inlineStr">
+      <c r="F103" s="30" t="inlineStr">
         <is>
           <t>KUMC: 不需要:MHSA 按项目整体录取(⚠️ 推断)
 Georgia State: 不需要:职业型项目(⚠️ 推断)
@@ -6230,32 +6573,32 @@
           <t>MA 生'通常获 1-4 学期支持';TA/RA 10-20 hr 含津贴+学费减免</t>
         </is>
       </c>
-      <c r="F107" s="29" t="inlineStr">
+      <c r="F107" s="30" t="inlineStr">
         <is>
           <t>⚠️ 官网未明确要求;建议:可先邮件联系研究方向匹配的教授,个人陈述中写明感兴趣的教授</t>
         </is>
       </c>
-      <c r="G107" s="29" t="inlineStr">
+      <c r="G107" s="30" t="inlineStr">
         <is>
           <t>可以申请(国际生可获TA/RA,但当TA需另证口语:TOEFL口语≥22/IELTS口语≥7.0/PTE口语≥75)。先修:区域认证学士学位,官网未列必修先修课;⚠️ 第三方称GPA 3.0为常见门槛。材料:CV、个人陈述(750–1000词)、3封推荐信</t>
         </is>
       </c>
-      <c r="H107" s="29" t="inlineStr">
+      <c r="H107" s="30" t="inlineStr">
         <is>
           <t>大学fellowship 2026/12/15;系assistantship 2027/1/31;1/31后仍审但资助优先级降低;不需资助者可申请周期外审核(⚠️ 按往年周期,2027待确认)</t>
         </is>
       </c>
-      <c r="I107" s="29" t="inlineStr">
+      <c r="I107" s="30" t="inlineStr">
         <is>
           <t>不需要(系官网:GRE no longer required)</t>
         </is>
       </c>
-      <c r="J107" s="29" t="inlineStr">
+      <c r="J107" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免):在美国院校完成≥30本科学分且GPA≥3.0即免TOEFL/IELTS(⚠️ 政策文件为2019–2020版);但当TA仍需证明口语(TOEFL口语≥22/IELTS口语≥7.0/PTE口语≥75或校内口语测试)</t>
         </is>
       </c>
-      <c r="K107" s="29" t="inlineStr">
+      <c r="K107" s="30" t="inlineStr">
         <is>
           <t>nathaniel.trumbull@uconn.edu(研究生项目协调员,⚠️ 系目录另列 debarchana.ghosh@uconn.edu 为协调员);gscu@uconn.edu(系办公室)</t>
         </is>
@@ -6292,32 +6635,32 @@
           <t>'硕士与博士级有限 assistantship';硕士最多 2 年</t>
         </is>
       </c>
-      <c r="F108" s="29" t="inlineStr">
+      <c r="F108" s="30" t="inlineStr">
         <is>
           <t>建议:系官网设有"Which Faculty Members are Accepting New Students?"页面,建议先确认在招导师并联系</t>
         </is>
       </c>
-      <c r="G108" s="29" t="inlineStr">
+      <c r="G108" s="30" t="inlineStr">
         <is>
           <t>可以申请(有限assistantship,⚠️ 官网未明确国际生限制)。注意:官方目录为 Geography M.S.(非MA)。先修:区域认证学士,GPA≥2.75;材料:成绩单、简历、goal statement、3封推荐信;⚠️ Peterson's称需相当于地理辅修(24学分)、建议GPA≥3.3</t>
         </is>
       </c>
-      <c r="H108" s="29" t="inlineStr">
+      <c r="H108" s="30" t="inlineStr">
         <is>
           <t>秋季优先截止 2027/2/1(材料齐全者最受优先考虑;按2025-26目录,2027待确认)</t>
         </is>
       </c>
-      <c r="I108" s="29" t="inlineStr">
+      <c r="I108" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不明确:官方目录招生要求未列GRE(大概率不需要);Peterson's 信息互相矛盾,建议邮件确认</t>
         </is>
       </c>
-      <c r="J108" s="29" t="inlineStr">
+      <c r="J108" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不明确(大概率否):Kent 要求"教育主要在美国以外"者提供英语证明,美本应可豁免,但未明文列出美国学位豁免,豁免需书面向国际招生办申请。不豁免时:TOEFL≥79,IELTS≥6.5,PTE≥58,DET≥110</t>
         </is>
       </c>
-      <c r="K108" s="29" t="inlineStr">
+      <c r="K108" s="30" t="inlineStr">
         <is>
           <t>ssmiley8@kent.edu(⚠️ 目录所列项目联系人 Sarah Smiley);geography@kent.edu(地理系办公室)</t>
         </is>
@@ -6354,32 +6697,32 @@
           <t>有限 assistantship;获资助者保证 4 学期(学费+津贴+医保补贴)</t>
         </is>
       </c>
-      <c r="F109" s="29" t="inlineStr">
+      <c r="F109" s="30" t="inlineStr">
         <is>
           <t>强烈建议:官网称录取很看重导师匹配,申请前联系潜在导师(建议8–9月),网申需填写意向教授</t>
         </is>
       </c>
-      <c r="G109" s="29" t="inlineStr">
+      <c r="G109" s="30" t="inlineStr">
         <is>
           <t>可以申请(有限assistantship,获资助者保证4学期;⚠️ 官网未明确限制国际生)。先修:学士学位,官网未列必修先修课;材料:CV、成绩单、letter of intent(约1500–2000词,≤3页单倍行距)、2封推荐信(第3封及≤15页写作样本可选)、申请费$50</t>
         </is>
       </c>
-      <c r="H109" s="29" t="inlineStr">
+      <c r="H109" s="30" t="inlineStr">
         <is>
           <t>最终 2026/12/1(2027秋季,Graduate School官网);春季入学仅特殊情况,需先联系研究生主任</t>
         </is>
       </c>
-      <c r="I109" s="29" t="inlineStr">
+      <c r="I109" s="30" t="inlineStr">
         <is>
           <t>不接受(官网:请勿提交GRE,委员会不审阅)</t>
         </is>
       </c>
-      <c r="J109" s="29" t="inlineStr">
+      <c r="J109" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不明确(大概率否):Graduate School 要求在非英语官方国家获英文授课学位者提交成绩,美国学位不在此列;但系有权自行要求。不豁免时:TOEFL≥80(2026/1/21后新版≥4.0)、IELTS≥6.5、PTE≥53、DET≥120</t>
         </is>
       </c>
-      <c r="K109" s="29" t="inlineStr">
+      <c r="K109" s="30" t="inlineStr">
         <is>
           <t>cnagel@mailbox.sc.edu(研究生主任 Caroline Nagel);nickless@mailbox.sc.edu(学生服务协调员 Sena Nickles)</t>
         </is>
@@ -7028,16 +7371,32 @@
           <t>全职GA 30学分学费减免+州外减免+stipend</t>
         </is>
       </c>
-      <c r="F126" s="21" t="n"/>
-      <c r="G126" s="21" t="inlineStr">
-        <is>
-          <t>可</t>
-        </is>
-      </c>
-      <c r="H126" s="21" t="n"/>
-      <c r="I126" s="21" t="n"/>
+      <c r="F126" s="30" t="inlineStr">
+        <is>
+          <t>不需要:无单独系内申请,经研究生院申请后选Urban Planning;GA职位建议主动联系项目主任</t>
+        </is>
+      </c>
+      <c r="G126" s="30" t="inlineStr">
+        <is>
+          <t>可以申请。先修:无指定本科专业;系要求本科GPA≥3.0,2.75–3.0可试读录取(前9学分需≥3.0);材料:成绩单、简历、300–500字目的陈述。另有PAB认证本科生36学分快轨</t>
+        </is>
+      </c>
+      <c r="H126" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 官网未列明确截止:材料须在开学前至少两周送达研究生院;资助/assistantship 3/1(第三方及手册提及,建议2027/3/1前提交);建议邮件确认</t>
+        </is>
+      </c>
+      <c r="I126" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 官网未提及GRE要求(手册录取标准未列考试),大概率不需要,建议确认</t>
+        </is>
+      </c>
       <c r="J126" s="21" t="n"/>
-      <c r="K126" s="21" t="n"/>
+      <c r="K126" s="30" t="inlineStr">
+        <is>
+          <t>planning@bsu.edu(城市规划系);admissions@bsu.edu(学校招生办)</t>
+        </is>
+      </c>
       <c r="L126" s="21" t="inlineStr">
         <is>
           <t>https://www.bsu.edu/academics/collegesanddepartments/urban-planning/applications-financial-aid/graduate-assistantships</t>
@@ -7070,32 +7429,32 @@
           <t>GA 10h/周含学费减免+医保补贴;二年级Public Service Assistantship</t>
         </is>
       </c>
-      <c r="F127" s="29" t="inlineStr">
+      <c r="F127" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,GA由系里分配;SOP可写感兴趣的教授/方向</t>
         </is>
       </c>
-      <c r="G127" s="29" t="inlineStr">
+      <c r="G127" s="30" t="inlineStr">
         <is>
           <t>可以申请(⚠️ 国际生GA资格官网未明文,建议确认)。需四年制学士学位、学术记录良好,不限本科专业;材料:非官方成绩单、3封推荐信(≥1封教授)、简历、≤1000字SOP。⚠️ 第三方称最低GPA 3.0</t>
         </is>
       </c>
-      <c r="H127" s="29" t="inlineStr">
+      <c r="H127" s="30" t="inlineStr">
         <is>
           <t>滚动录取,2027/1/15起开始审理(按2026-27手册);建议 2027/3/1 前提交以优先考虑系里assistantship</t>
         </is>
       </c>
-      <c r="I127" s="29" t="inlineStr">
+      <c r="I127" s="30" t="inlineStr">
         <is>
           <t>不需要(官网标注 GRE Waived)</t>
         </is>
       </c>
-      <c r="J127" s="29" t="inlineStr">
+      <c r="J127" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免):Clemson研究生院对美国区域认证院校学位豁免ELP,在读学位可先获豁免、入学前补交学位成绩单。否则 TOEFL ≥80(项目偏好100)/IELTS ≥6.5/Duolingo ≥115</t>
         </is>
       </c>
-      <c r="K127" s="29" t="inlineStr">
+      <c r="K127" s="30" t="inlineStr">
         <is>
           <t>mcrp@clemson.edu(MCRP项目邮箱);grdapp@clemson.edu(研究生院招生)</t>
         </is>
@@ -7132,27 +7491,27 @@
           <t>'TAships and GRships include a stipend and a full waiver of base tuition';'All graduate applicants (domestic and international) are automatically considered'</t>
         </is>
       </c>
-      <c r="F128" s="29" t="inlineStr">
+      <c r="F128" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,所有申请者(含国际生)自动考虑TA/GR</t>
         </is>
       </c>
-      <c r="G128" s="29" t="inlineStr">
+      <c r="G128" s="30" t="inlineStr">
         <is>
           <t>可以申请(国际生同样自动考虑TA/GR,含stipend+基础学费全免)。不限本科专业;⚠️ 第三方称最低GPA 3.0;TOEFL ≥80/IELTS ≥6.5(如需)</t>
         </is>
       </c>
-      <c r="H128" s="29" t="inlineStr">
+      <c r="H128" s="30" t="inlineStr">
         <is>
           <t>录取+资助优先 2027/1/10;⚠️ 系页面称晚申请可至 2/1;最终:国际生 6/1、国内 7/1(按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I128" s="29" t="inlineStr">
+      <c r="I128" s="30" t="inlineStr">
         <is>
           <t>不需要(可选提交,须截止前送达;校代码4853/系代码4402)</t>
         </is>
       </c>
-      <c r="J128" s="29" t="inlineStr">
+      <c r="J128" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免,有条件):美国区域认证学士学位须在提交申请并缴费前2年内获得;否则 TOEFL ≥80/IELTS ≥6.5/Duolingo ≥110</t>
         </is>
@@ -7190,23 +7549,23 @@
           <t>merit aid(assistantships/fellowships/tuition remission)需1/15前申请;'Funds will only cover a portion of all applicants'</t>
         </is>
       </c>
-      <c r="F129" s="29" t="inlineStr">
+      <c r="F129" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,奖学金/assistantship由学院综合评审分配</t>
         </is>
       </c>
       <c r="G129" s="21" t="n"/>
-      <c r="H129" s="29" t="inlineStr">
+      <c r="H129" s="30" t="inlineStr">
         <is>
           <t>资助优先 2027/1/15(按2026周期,2027待公布);⚠️ 最终(2026周期program explorer):国际生 4/1、美国申请者 7/1;春季 11/1</t>
         </is>
       </c>
-      <c r="I129" s="29" t="inlineStr">
+      <c r="I129" s="30" t="inlineStr">
         <is>
           <t>不需要(近几个周期均对所有申请者 waive)</t>
         </is>
       </c>
-      <c r="J129" s="29" t="inlineStr">
+      <c r="J129" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不明确:Bloustein项目列表写 Non-U.S. applicants 需 TOEFL/IELTS/Duolingo,未写美国学位豁免;研究生院部分项目对≥3年英语授课本科豁免,建议邮件确认</t>
         </is>
@@ -7244,27 +7603,27 @@
           <t>'limited number of graduate assistantships on a competitive basis';考虑截止3/1</t>
         </is>
       </c>
-      <c r="F130" s="29" t="inlineStr">
+      <c r="F130" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,GA有限且竞争性分配</t>
         </is>
       </c>
-      <c r="G130" s="29" t="inlineStr">
+      <c r="G130" s="30" t="inlineStr">
         <is>
           <t>可以申请(GA名额有限、竞争性)。研究生院最低GPA 3.0(低于者可凭工作经历等综合考虑);不限本科专业;材料:成绩单、个人陈述、简历、3封推荐信</t>
         </is>
       </c>
-      <c r="H130" s="29" t="inlineStr">
+      <c r="H130" s="30" t="inlineStr">
         <is>
           <t>GA/资助优先 2027/3/1(春季入学 10/1);最终滚动截止:秋季 8/1、春季 1/1</t>
         </is>
       </c>
-      <c r="I130" s="29" t="inlineStr">
+      <c r="I130" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不需要:现行FAQ未提GRE;旧版FAQ仅要求非美国本科者提交GRE(美本不受影响)</t>
         </is>
       </c>
-      <c r="J130" s="29" t="inlineStr">
+      <c r="J130" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免):已获英语授课认可院校学位者豁免;否则 TOEFL iBT ≥90(各部分≥20)/IELTS ≥6.5。⚠️ 豁免措辞为'已获得'学位,在读者建议确认</t>
         </is>
@@ -7302,12 +7661,36 @@
           <t>Wilder Graduate Scholars Fellowship:州内学费杂费+stipend(2024-25共$32,752),1年,24个名额跨4项目;国际生资格未明</t>
         </is>
       </c>
-      <c r="F131" s="21" t="n"/>
-      <c r="G131" s="21" t="n"/>
-      <c r="H131" s="21" t="n"/>
-      <c r="I131" s="21" t="n"/>
-      <c r="J131" s="21" t="n"/>
-      <c r="K131" s="21" t="n"/>
+      <c r="F131" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取,个人陈述可写感兴趣方向</t>
+        </is>
+      </c>
+      <c r="G131" s="30" t="inlineStr">
+        <is>
+          <t>可以申请,但Wilder Graduate Scholars Fellowship国际生资格未明。先修:无指定专业;本科GPA≥2.7(4.0制),低于可试读录取;3封推荐信,至少2封来自教师</t>
+        </is>
+      </c>
+      <c r="H131" s="30" t="inlineStr">
+        <is>
+          <t>早申/优先 2027/2/1;目录另列秋季优先 4/1;最终 2027/5/1(按Wilder官网周期推算,2027待确认);逾期可交但不保证审理</t>
+        </is>
+      </c>
+      <c r="I131" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 不明确:官方目录测试要求栏未能读取,第三方称需GRE但可能过时,建议邮件确认</t>
+        </is>
+      </c>
+      <c r="J131" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 不明确:VCU研究生豁免列表所列国家未能确认含美国;否则需 TOEFL iBT ≥80(2026/1/21后新制≥4.5)/ IELTS ≥6.5,2年有效,建议确认</t>
+        </is>
+      </c>
+      <c r="K131" s="30" t="inlineStr">
+        <is>
+          <t>wsrecruit@vcu.edu(Wilder School招生/招募)</t>
+        </is>
+      </c>
       <c r="L131" s="21" t="inlineStr">
         <is>
           <t>https://wilder.vcu.edu/student-support-resources/internships-and-experiential-learning-/wilder-graduate-scholars-fellowship/</t>
@@ -7340,12 +7723,36 @@
           <t>TA/RA'cover tuition, plus a stipend'</t>
         </is>
       </c>
-      <c r="F132" s="21" t="n"/>
-      <c r="G132" s="21" t="n"/>
-      <c r="H132" s="21" t="n"/>
-      <c r="I132" s="21" t="n"/>
-      <c r="J132" s="21" t="n"/>
-      <c r="K132" s="21" t="n"/>
+      <c r="F132" s="30" t="inlineStr">
+        <is>
+          <t>建议:研究型MS(可写论文),官网要求申请人先阅读研究生手册并联系Graduate Chair Dr. Harold Perkins</t>
+        </is>
+      </c>
+      <c r="G132" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(TA/RA可覆盖学费+stipend;资助仅限秋季入学)。先修:接受非地理专业,但需在个人陈述说明本科如何为地理研究生学习做准备;资助/无条件录取一般需GPA≥3.0;1–2页陈述、简历、3封推荐信</t>
+        </is>
+      </c>
+      <c r="H132" s="30" t="inlineStr">
+        <is>
+          <t>资助截止 2027/1/15(申请窗口 2026/10/15–2027/1/15);一般2月审理,3/15前通知</t>
+        </is>
+      </c>
+      <c r="I132" s="30" t="inlineStr">
+        <is>
+          <t>不需要(系官网明确GRE not required)</t>
+        </is>
+      </c>
+      <c r="J132" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免):OU规定来自非英语国家者须在入学前2年内获得美国区域认证院校学士学位才可豁免;否则 ⚠️ TOEFL 80 / IELTS 6.5(第三方)。当TA可能另有口语要求,建议确认</t>
+        </is>
+      </c>
+      <c r="K132" s="30" t="inlineStr">
+        <is>
+          <t>perkinsh@ohio.edu(Graduate Chair Dr. Harold Perkins)</t>
+        </is>
+      </c>
       <c r="L132" s="21" t="inlineStr">
         <is>
           <t>https://www.ohio.edu/cas/geography/graduate/financial-aid</t>
@@ -7378,12 +7785,36 @@
           <t>'eligible for GRA and TA positions after their first semester';$300k+奖学金/年</t>
         </is>
       </c>
-      <c r="F133" s="21" t="n"/>
-      <c r="G133" s="21" t="n"/>
-      <c r="H133" s="21" t="n"/>
-      <c r="I133" s="21" t="n"/>
-      <c r="J133" s="21" t="n"/>
-      <c r="K133" s="21" t="n"/>
+      <c r="F133" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取,个人陈述可写感兴趣教授/方向</t>
+        </is>
+      </c>
+      <c r="G133" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(第一学期后可申GRA/TA)。先修:无指定本科专业;1000–1500字目的陈述,另可提交可选写作样本</t>
+        </is>
+      </c>
+      <c r="H133" s="30" t="inlineStr">
+        <is>
+          <t>2027/1/3 10:59PM CST(官网,仅秋季入学);⚠️ 第三方列2026/12/15,以官网为准</t>
+        </is>
+      </c>
+      <c r="I133" s="30" t="inlineStr">
+        <is>
+          <t>不需要(MSCRP已永久免GRE)</t>
+        </is>
+      </c>
+      <c r="J133" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免):UT研究生院豁免持美国院校学士学位者;否则 TOEFL ≥79 / IELTS ≥6.5 / DET ≥115</t>
+        </is>
+      </c>
+      <c r="K133" s="30" t="inlineStr">
+        <is>
+          <t>soa_grad@austin.utexas.edu(建筑学院研究生招生办);CRP-advisor@austin.utexas.edu(MSCRP研究生顾问)</t>
+        </is>
+      </c>
       <c r="L133" s="21" t="inlineStr">
         <is>
           <t>https://soa.utexas.edu/apply/financial-support</t>
@@ -7416,16 +7847,36 @@
           <t>'Both US and non-US citizens are eligible for merit-based scholarships';委员会审核时分配</t>
         </is>
       </c>
-      <c r="F134" s="21" t="n"/>
+      <c r="F134" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取,委员会审核时分配奖学金</t>
+        </is>
+      </c>
       <c r="G134" s="21" t="inlineStr">
         <is>
           <t>可</t>
         </is>
       </c>
-      <c r="H134" s="21" t="n"/>
-      <c r="I134" s="21" t="n"/>
-      <c r="J134" s="21" t="n"/>
-      <c r="K134" s="21" t="n"/>
+      <c r="H134" s="30" t="inlineStr">
+        <is>
+          <t>2027/1/13 11:59PM ET(Weitzman官网,2027秋季MCP)</t>
+        </is>
+      </c>
+      <c r="I134" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 不明确:How to Apply页仍将MCP列入标准化考试要求(5年有效),旧页面曾称Fall 2023免GRE;建议按需提交或邮件确认</t>
+        </is>
+      </c>
+      <c r="J134" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免):Weitzman规定本科≥4年非英语授课者才需提交;美国本科英语授课无需提交。如需提交仅接受 TOEFL/IELTS/Duolingo</t>
+        </is>
+      </c>
+      <c r="K134" s="30" t="inlineStr">
+        <is>
+          <t>admissions@design.upenn.edu(Weitzman招生办);cityplan@design.upenn.edu(城市与区域规划系)</t>
+        </is>
+      </c>
       <c r="L134" s="21" t="inlineStr">
         <is>
           <t>https://www.design.upenn.edu/graduate-admissions/tuition-and-financial-aid</t>
@@ -7458,16 +7909,32 @@
           <t>'GE awards include a full tuition waiver, health insurance, and a competitive monthly stipend';'approximately 30 terms of GE positions per year'(≈10个全年,跨MCRP/MPA/MNM);优先2/1</t>
         </is>
       </c>
-      <c r="F135" s="21" t="n"/>
-      <c r="G135" s="21" t="inlineStr">
-        <is>
-          <t>可</t>
-        </is>
-      </c>
-      <c r="H135" s="21" t="n"/>
-      <c r="I135" s="21" t="n"/>
+      <c r="F135" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取;可参加线上信息会(2026/11/13、2027/1/15)</t>
+        </is>
+      </c>
+      <c r="G135" s="30" t="inlineStr">
+        <is>
+          <t>可以申请(GE含全额学费减免+医保+月薪)。先修:无指定专业;需修过高年级本科或研究生入门统计(可作PPPM 613前置/同修,相当课程或工作经验可豁免);3封推荐信</t>
+        </is>
+      </c>
+      <c r="H135" s="30" t="inlineStr">
+        <is>
+          <t>优先 2027/2/1;最终 2027/8/15(太平洋时间23:59);逾期视名额接收</t>
+        </is>
+      </c>
+      <c r="I135" s="30" t="inlineStr">
+        <is>
+          <t>可选(提交则综合考虑,也接受GMAT)</t>
+        </is>
+      </c>
       <c r="J135" s="21" t="n"/>
-      <c r="K135" s="21" t="n"/>
+      <c r="K135" s="30" t="inlineStr">
+        <is>
+          <t>choquett@uoregon.edu(研究生协调员Bob Choquette);abrown33@uoregon.edu(MCRP主任Anne Brown)</t>
+        </is>
+      </c>
       <c r="L135" s="21" t="inlineStr">
         <is>
           <t>https://pppm.uoregon.edu/grad/funding</t>
@@ -7500,12 +7967,32 @@
           <t>GA:≥9学分学费减免+部分fee+月stipend;PPDA两年承诺(学费≤36学分/年+时薪)每届约2人</t>
         </is>
       </c>
-      <c r="F136" s="21" t="n"/>
+      <c r="F136" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取;可预约与MURP主任一对一交流</t>
+        </is>
+      </c>
       <c r="G136" s="21" t="n"/>
-      <c r="H136" s="21" t="n"/>
-      <c r="I136" s="21" t="n"/>
-      <c r="J136" s="21" t="n"/>
-      <c r="K136" s="21" t="n"/>
+      <c r="H136" s="30" t="inlineStr">
+        <is>
+          <t>优先 2026/1/9;第二轮 3/27;第三轮 5/29(补充材料各轮后一周)(按2026周期,2027待公布)</t>
+        </is>
+      </c>
+      <c r="I136" s="30" t="inlineStr">
+        <is>
+          <t>不接受(自Fall 2021起GRE不再纳入审核)</t>
+        </is>
+      </c>
+      <c r="J136" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 否(美国学位豁免):PSU研究生英语要求页(ondeck子域)列美国学士学位为有效证明;否则 TOEFL ≥80(2年内)</t>
+        </is>
+      </c>
+      <c r="K136" s="30" t="inlineStr">
+        <is>
+          <t>murpadm@pdx.edu(MURP招生);⚠️ askusp@pdx.edu(第三方列出)</t>
+        </is>
+      </c>
       <c r="L136" s="21" t="inlineStr">
         <is>
           <t>https://www.pdx.edu/urban-studies-planning/financial-resources</t>
@@ -7538,16 +8025,36 @@
           <t>Full line=20h/周+9学分学费+stipend;资助截止3/15;研究生院明文国际生可获系管奖学金与assistantship</t>
         </is>
       </c>
-      <c r="F137" s="21" t="n"/>
+      <c r="F137" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取</t>
+        </is>
+      </c>
       <c r="G137" s="21" t="inlineStr">
         <is>
           <t>可</t>
         </is>
       </c>
-      <c r="H137" s="21" t="n"/>
-      <c r="I137" s="21" t="n"/>
-      <c r="J137" s="21" t="n"/>
-      <c r="K137" s="21" t="n"/>
+      <c r="H137" s="30" t="inlineStr">
+        <is>
+          <t>资助截止 2027/3/15(仅秋季);⚠️ 非资助申请可能为滚动录取(据MRP/JD页,建议3/15前提交)</t>
+        </is>
+      </c>
+      <c r="I137" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 可能不需要:第三方称独立MRP无GRE要求,官网未确认</t>
+        </is>
+      </c>
+      <c r="J137" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免):在美国院校完成≥4个全日制学期且平均≥B可申请豁免(研究生院评估);否则 ⚠️ TOEFL 79 / IELTS 6.5 / Duolingo 110 / PTE 53</t>
+        </is>
+      </c>
+      <c r="K137" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ lawsonc@albany.edu(Regional Planning研究生主任Catherine Lawson,邮箱来自旧页面,建议核实)</t>
+        </is>
+      </c>
       <c r="L137" s="21" t="inlineStr">
         <is>
           <t>https://www.albany.edu/geographyplanning/programs/mrp-urban-and-regional-planning</t>
@@ -7580,12 +8087,28 @@
           <t>两年RA(stipend+24学分学费)限BIPOC/Hispanic GPA≥3.5;FDOT Transit Fellow一年stipend+全额学费;系资助申请2/15</t>
         </is>
       </c>
-      <c r="F138" s="21" t="n"/>
+      <c r="F138" s="30" t="inlineStr">
+        <is>
+          <t>不需要:按项目整体录取,滚动审理</t>
+        </is>
+      </c>
       <c r="G138" s="21" t="n"/>
-      <c r="H138" s="21" t="n"/>
-      <c r="I138" s="21" t="n"/>
+      <c r="H138" s="30" t="inlineStr">
+        <is>
+          <t>系资助 2027/2/15;国际生秋季 2027/1/15(⚠️ 页面正文另写6/1,冲突);美国申请者 7/1;滚动录取</t>
+        </is>
+      </c>
+      <c r="I138" s="30" t="inlineStr">
+        <is>
+          <t>不需要(MSP暂免GRE)</t>
+        </is>
+      </c>
       <c r="J138" s="21" t="n"/>
-      <c r="K138" s="21" t="n"/>
+      <c r="K138" s="30" t="inlineStr">
+        <is>
+          <t>durp@coss.fsu.edu(DURP招生协调员)</t>
+        </is>
+      </c>
       <c r="L138" s="21" t="inlineStr">
         <is>
           <t>https://cosspp.fsu.edu/durp/Admissions/</t>
@@ -7618,12 +8141,32 @@
           <t>Irving Harris MCH Scholars:每年 3 个新生获学费减免+月津贴(一年级秋春);MCH MPH Scholars 2/yr $2,000-5,000</t>
         </is>
       </c>
-      <c r="F139" s="21" t="n"/>
+      <c r="F139" s="30" t="inlineStr">
+        <is>
+          <t>不需要:SOPHAS统一申请,按项目整体录取</t>
+        </is>
+      </c>
       <c r="G139" s="21" t="n"/>
-      <c r="H139" s="21" t="n"/>
-      <c r="I139" s="21" t="n"/>
-      <c r="J139" s="21" t="n"/>
-      <c r="K139" s="21" t="n"/>
+      <c r="H139" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 官网冲突:MCH页写国际生 2026/12/15、国内 2027/2/1;SPH总页写资助优先 12/1、国际生 2/1、最终 4/15;建议12/1前提交</t>
+        </is>
+      </c>
+      <c r="I139" s="30" t="inlineStr">
+        <is>
+          <t>可选(提交会被考虑,代码7931)</t>
+        </is>
+      </c>
+      <c r="J139" s="30" t="inlineStr">
+        <is>
+          <t>否(美国学位豁免):UIC豁免近5年内在美国认证院校全日制学习≥2年者;否则 TOEFL iBT 80(新制4.5)/ IELTS 6.5 / PTE 54</t>
+        </is>
+      </c>
+      <c r="K139" s="30" t="inlineStr">
+        <is>
+          <t>sph-admissions@uic.edu(公卫学院招生);jacobw@uic.edu(招生助理主任Jacob Wilson)</t>
+        </is>
+      </c>
       <c r="L139" s="21" t="inlineStr">
         <is>
           <t>https://maternalchild.uic.edu/admissions/financial-aid-and-scholarships</t>
@@ -7930,28 +8473,28 @@
           <t>TA/RA/work-study多渠道;无学费减免说明</t>
         </is>
       </c>
-      <c r="F147" s="29" t="inlineStr">
+      <c r="F147" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取;个人陈述中写明研究兴趣与感兴趣的教师即可</t>
         </is>
       </c>
-      <c r="G147" s="29" t="inlineStr">
+      <c r="G147" s="30" t="inlineStr">
         <is>
           <t>可以申请(资助为TA/RA/work-study,未见学费减免说明)。需学士学位,总GPA≥3.0;心理学专业或具足够心理学背景(大学数学、统计、实验心理学及生物/物理/社会科学基础);非心理专业建议补统计、研究方法、认知、生理心理、社会心理等;未完全达标的优秀者也可被考虑</t>
         </is>
       </c>
-      <c r="H147" s="29" t="inlineStr">
+      <c r="H147" s="30" t="inlineStr">
         <is>
           <t>2026/12/15(系FAQ:全部材料截止,次年秋季入学);⚠️ 校目录(2025/6)写1/1,以系网站为准</t>
         </is>
       </c>
-      <c r="I147" s="29" t="inlineStr">
+      <c r="I147" s="30" t="inlineStr">
         <is>
           <t>不需要(系FAQ明确不要求;旧手册写可选)</t>
         </is>
       </c>
       <c r="J147" s="21" t="n"/>
-      <c r="K147" s="29" t="inlineStr">
+      <c r="K147" s="30" t="inlineStr">
         <is>
           <t>alac@uccs.edu(Andrew Lac,Psychological Science培养主任);intladms@uccs.edu(国际生招生)</t>
         </is>
@@ -7988,32 +8531,32 @@
           <t>校级GA:tuition remission+月薪+医保;硕士≤4学期</t>
         </is>
       </c>
-      <c r="F148" s="29" t="inlineStr">
+      <c r="F148" s="30" t="inlineStr">
         <is>
           <t>建议:研究型MA(Plan A论文),个人陈述写明匹配教师;官网未要求申请前联系</t>
         </is>
       </c>
-      <c r="G148" s="29" t="inlineStr">
+      <c r="G148" s="30" t="inlineStr">
         <is>
           <t>可以申请(校级GA含学费减免+月薪+医保)。学士学位GPA≥3.0;≥15学分心理学课程,须含基础统计、高年级实验课,以及以实验方法为主的独立研究(数据收集、统计分析、报告写作);方向:Cognitive/Developmental/Neuroscience &amp; Behavior</t>
         </is>
       </c>
-      <c r="H148" s="29" t="inlineStr">
+      <c r="H148" s="30" t="inlineStr">
         <is>
           <t>1/10(按2026周期为2026/1/10,2027待公布)</t>
         </is>
       </c>
-      <c r="I148" s="29" t="inlineStr">
+      <c r="I148" s="30" t="inlineStr">
         <is>
           <t>可选:提交与否均审核</t>
         </is>
       </c>
-      <c r="J148" s="29" t="inlineStr">
+      <c r="J148" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免);否则 TOEFL iBT ≥80,IELTS ≥6.5,PTE ≥53,Duolingo ≥110</t>
         </is>
       </c>
-      <c r="K148" s="29" t="inlineStr">
+      <c r="K148" s="30" t="inlineStr">
         <is>
           <t>unopsycgrad@unomaha.edu(心理系研究生项目)</t>
         </is>
@@ -8050,27 +8593,27 @@
           <t>GIA岗位需按优先截止申请;GTA限二年级;GRA看导师经费</t>
         </is>
       </c>
-      <c r="F149" s="29" t="inlineStr">
+      <c r="F149" s="30" t="inlineStr">
         <is>
           <t>建议:申请材料须按偏好列出3位匹配教师(研究兴趣声明);GRA看导师经费,可提前邮件联系</t>
         </is>
       </c>
-      <c r="G149" s="29" t="inlineStr">
+      <c r="G149" s="30" t="inlineStr">
         <is>
           <t>可以申请(GIA岗位需按优先截止申请;GTA限二年级)。GPA≥3.0;心理学导论、统计、实验/研究方法(或相关学科)须B及以上;需研究兴趣声明、简历/CV、1-2页个人陈述;国际学历申请费$90</t>
         </is>
       </c>
-      <c r="H149" s="29" t="inlineStr">
+      <c r="H149" s="30" t="inlineStr">
         <is>
           <t>资助优先 2026/2/1;最终 2026/4/30(按2026周期,2027待公布);仅秋季入学</t>
         </is>
       </c>
-      <c r="I149" s="29" t="inlineStr">
+      <c r="I149" s="30" t="inlineStr">
         <is>
           <t>不需要(明确不纳入录取考虑)</t>
         </is>
       </c>
-      <c r="J149" s="29" t="inlineStr">
+      <c r="J149" s="30" t="inlineStr">
         <is>
           <t>否(美国区域认证学士学位豁免);否则 TOEFL iBT ≥78(2026/1/21前考试的标准,新分制下要求待确认)</t>
         </is>
@@ -8732,27 +9275,27 @@
           <t>GA薪资表:MS $18,348–27,800/yr,Tuition Waiver: YES;由导师发布岗位</t>
         </is>
       </c>
-      <c r="F166" s="29" t="inlineStr">
+      <c r="F166" s="30" t="inlineStr">
         <is>
           <t>强烈建议:官网要求先匹配兴趣相符的教师并获其支持作为major professor;GA岗位多由导师发布</t>
         </is>
       </c>
-      <c r="G166" s="29" t="inlineStr">
+      <c r="G166" s="30" t="inlineStr">
         <is>
           <t>可以申请。先修:欢迎林业、渔业、野生动物及其他背景,背景不符可能需补课;硕士最低本科GPA 3.0。TA另需符合UGA TA英语政策</t>
         </is>
       </c>
-      <c r="H166" s="29" t="inlineStr">
+      <c r="H166" s="30" t="inlineStr">
         <is>
           <t>Graduate School助教金截止 12/1(建议 2026/12/1 前完成申请以竞争资助);最终截止:国际生 4/15、国内 7/1(按官网常规日期,2027待核实)</t>
         </is>
       </c>
-      <c r="I166" s="29" t="inlineStr">
+      <c r="I166" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不明确:Warnell助研岗位注明不需要GRE;Peterson's(第三方)仍列GRE,建议邮件确认</t>
         </is>
       </c>
-      <c r="J166" s="29" t="inlineStr">
+      <c r="J166" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免):UGA研究生院规定美国认证大学学位一般免交TOEFL/IELTS(个别项目可另要求);如需:TOEFL 80(各项≥20)/IELTS 6.5;当TA另有英语要求</t>
         </is>
@@ -8790,32 +9333,32 @@
           <t>'limited number of assistantships on a competitive basis';MS stipend $16,500/yr+全额学费减免(自付fees)</t>
         </is>
       </c>
-      <c r="F167" s="29" t="inlineStr">
+      <c r="F167" s="30" t="inlineStr">
         <is>
           <t>必须:SRNR录取要求申请时已确定major professor,建议先联系导师确认岗位</t>
         </is>
       </c>
-      <c r="G167" s="29" t="inlineStr">
+      <c r="G167" s="30" t="inlineStr">
         <is>
           <t>可以申请(资助为竞争性少量assistantship)。先修:认证大学学士学位,需获项目51%研究生教师认可并有确定导师;成功申请者一般GPA≥3.25、GRE V+Q≥300</t>
         </is>
       </c>
-      <c r="H167" s="29" t="inlineStr">
+      <c r="H167" s="30" t="inlineStr">
         <is>
           <t>⚠️ 研究生院历史资助优先日 1/25;国际生最终截止 5/1 或 5/15(LSU不同页面冲突),国内约 6/30–7/1;项目可能更早(按往年,2027待公布)</t>
         </is>
       </c>
-      <c r="I167" s="29" t="inlineStr">
+      <c r="I167" s="30" t="inlineStr">
         <is>
           <t>⚠️ 必需/参考:官网称成功申请者GRE V+Q一般≥300;Gilbert资助要求≥310,建议确认是否仍强制</t>
         </is>
       </c>
-      <c r="J167" s="29" t="inlineStr">
+      <c r="J167" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免):LSU规定持美国院校学士学位可免;如需:TOEFL 79,IELTS 6.5</t>
         </is>
       </c>
-      <c r="K167" s="29" t="inlineStr">
+      <c r="K167" s="30" t="inlineStr">
         <is>
           <t>⚠️ staylor@lsu.edu(研究生协调员 Dr. Sabrina Taylor,官网不同版本另列 wkelso@lsu.edu);gradadmission@lsu.edu(研究生院招生)</t>
         </is>
@@ -8852,28 +9395,28 @@
           <t>'application will not be reviewed until you and your future advisor have arrangements for funding';GRA经导师</t>
         </is>
       </c>
-      <c r="F168" s="29" t="inlineStr">
+      <c r="F168" s="30" t="inlineStr">
         <is>
           <t>必须:须有教师同意担任导师才会审理申请;thesis MS须与导师落实资助方案后才审</t>
         </is>
       </c>
-      <c r="G168" s="29" t="inlineStr">
+      <c r="G168" s="30" t="inlineStr">
         <is>
           <t>可以申请,但须先落实导师和资助(GRA经导师)。先修:⚠️ 官网未列具体先修课,建议咨询研究生顾问</t>
         </is>
       </c>
-      <c r="H168" s="29" t="inlineStr">
+      <c r="H168" s="30" t="inlineStr">
         <is>
           <t>奖学金提名 2026/12/31(需完成申请);国际生最终 2027/2/1;国内 2027/5/1</t>
         </is>
       </c>
       <c r="I168" s="21" t="n"/>
-      <c r="J168" s="29" t="inlineStr">
+      <c r="J168" s="30" t="inlineStr">
         <is>
           <t>否(美国学位豁免):TAMU规定持美国认证院校学士学位免交成绩(项目可另设更高要求);当TA需通过ELPE口语(≥80)或申请替代认证</t>
         </is>
       </c>
-      <c r="K168" s="29" t="inlineStr">
+      <c r="K168" s="30" t="inlineStr">
         <is>
           <t>⚠️ 官网邮箱未能读取:研究生学术顾问 Wenwen Zhou,电话979-314-5715,建议通过rwfm.tamu.edu/contact-advisor联系</t>
         </is>
@@ -8910,24 +9453,24 @@
           <t>入学时部分学费merit奖;GSI/GSRA含全额学费+医保+stipend但竞争性、多入学后申请</t>
         </is>
       </c>
-      <c r="F169" s="29" t="inlineStr">
+      <c r="F169" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取;GSRA多入学后申请,可在申请材料中提及感兴趣教授</t>
         </is>
       </c>
       <c r="G169" s="21" t="n"/>
-      <c r="H169" s="29" t="inlineStr">
+      <c r="H169" s="30" t="inlineStr">
         <is>
           <t>资助优先 2026/12/15;资助最终 2027/1/14;最终:国际生 2027/4/1,国内 2027/4/30</t>
         </is>
       </c>
-      <c r="I169" s="29" t="inlineStr">
+      <c r="I169" s="30" t="inlineStr">
         <is>
           <t>不接受(已不再要求也不接受GRE)</t>
         </is>
       </c>
       <c r="J169" s="21" t="n"/>
-      <c r="K169" s="29" t="inlineStr">
+      <c r="K169" s="30" t="inlineStr">
         <is>
           <t>⚠️ seas-admissions@umich.edu(SEAS招生,据记忆需核实);电话 (734) 764-6453</t>
         </is>
@@ -9666,28 +10209,28 @@
           <t>'Assistantships provide a tuition waiver and a stipend';硕士最多2年半时;non-thesis低优先</t>
         </is>
       </c>
-      <c r="F187" s="29" t="inlineStr">
+      <c r="F187" s="30" t="inlineStr">
         <is>
           <t>⚠️ 不需要(官网未要求):按项目整体录取;可在个人陈述中写方向匹配的教授,或先联系方向负责人(如犯罪学 Katie Constantin)</t>
         </is>
       </c>
-      <c r="G187" s="29" t="inlineStr">
+      <c r="G187" s="30" t="inlineStr">
         <is>
           <t>可以申请(助教/助研含学费减免+津贴,国际生可申)。先修:官网未列明最低GPA与必修先修课;项目核心为理论、方法、统计。材料:CV、3位推荐人、2-3页个人陈述、非正式成绩单,写作样本可选</t>
         </is>
       </c>
-      <c r="H187" s="29" t="inlineStr">
+      <c r="H187" s="30" t="inlineStr">
         <is>
           <t>资助优先 2027/2/1;秋季最终 2027/4/1(据系研究生手册2025年12月版;旧页面曾写4/15,2027待确认)</t>
         </is>
       </c>
-      <c r="I187" s="29" t="inlineStr">
+      <c r="I187" s="30" t="inlineStr">
         <is>
           <t>不需要(系申请页明确不再要求GRE)</t>
         </is>
       </c>
       <c r="J187" s="21" t="n"/>
-      <c r="K187" s="29" t="inlineStr">
+      <c r="K187" s="30" t="inlineStr">
         <is>
           <t>jonathan.s.coley@okstate.edu(研究生项目主任 Jonathan Coley);grad-i@okstate.edu(研究生院国际招生)</t>
         </is>
@@ -9724,7 +10267,7 @@
           <t>'All applicants are considered for funding';GA stipend $18,540/9月</t>
         </is>
       </c>
-      <c r="F188" s="29" t="inlineStr">
+      <c r="F188" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,所有申请者自动参与资助评审;目标陈述中写研究兴趣及与教师的匹配即可</t>
         </is>
@@ -9735,13 +10278,13 @@
         </is>
       </c>
       <c r="H188" s="21" t="n"/>
-      <c r="I188" s="29" t="inlineStr">
+      <c r="I188" s="30" t="inlineStr">
         <is>
           <t>不需要(自2026秋季入学起取消GRE;旧版2025-26目录仍写需要)</t>
         </is>
       </c>
       <c r="J188" s="21" t="n"/>
-      <c r="K188" s="29" t="inlineStr">
+      <c r="K188" s="30" t="inlineStr">
         <is>
           <t>sroxburg@kent.edu(研究生项目协调员 Susan Roxburgh);soc_crim@kent.edu(系办公室)</t>
         </is>
@@ -9778,7 +10321,7 @@
           <t>GA+学费杂费减免'including out-of-state or international tuition';通常2年</t>
         </is>
       </c>
-      <c r="F189" s="29" t="inlineStr">
+      <c r="F189" s="30" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取;个人陈述说明攻读社会学的原因与兴趣方向即可</t>
         </is>
@@ -9788,18 +10331,18 @@
           <t>可</t>
         </is>
       </c>
-      <c r="H189" s="29" t="inlineStr">
+      <c r="H189" s="30" t="inlineStr">
         <is>
           <t>GA资助优先 2027/3/1;最终:国际生 2027/5/1(秋季),国内 2027/7/1(按系官网现行日期,2027待确认)</t>
         </is>
       </c>
-      <c r="I189" s="29" t="inlineStr">
+      <c r="I189" s="30" t="inlineStr">
         <is>
           <t>不需要(系官网明确不要求GRE;Peterson's称需要,已过时)</t>
         </is>
       </c>
       <c r="J189" s="21" t="n"/>
-      <c r="K189" s="29" t="inlineStr">
+      <c r="K189" s="30" t="inlineStr">
         <is>
           <t>socgradcoord@memphis.edu(研究生项目邮箱);tmccuddy@memphis.edu(研究生主任 Timothy McCuddy)</t>
         </is>
@@ -10464,22 +11007,22 @@
           <t>'limited number of graduate assistantships…we cannot make any guarantees';'primarily awarded to doctoral students'</t>
         </is>
       </c>
-      <c r="F206" s="30" t="inlineStr">
+      <c r="F206" s="31" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,每年仅秋季入学一次;个人陈述可写感兴趣的教授</t>
         </is>
       </c>
-      <c r="G206" s="30" t="inlineStr">
+      <c r="G206" s="31" t="inlineStr">
         <is>
           <t>可以申请,但资助极少(系招生页称目前不为硕士生提供assistantship,GA主要给博士)。先修:美国认证大学学士学位;无指定专业先修课;需700–1200词个人陈述、3封推荐信、全部成绩单;⚠️ 最低GPA系页未写明(研究生院通常要求约2.75,建议确认)</t>
         </is>
       </c>
-      <c r="H206" s="30" t="inlineStr">
+      <c r="H206" s="31" t="inlineStr">
         <is>
           <t>2027/1/15(按系研究生手册2024–25所列每年1/15截止,2027待公布);每年仅秋季入学一次</t>
         </is>
       </c>
-      <c r="I206" s="30" t="inlineStr">
+      <c r="I206" s="31" t="inlineStr">
         <is>
           <t>不需要(系招生页明确不要求GRE)</t>
         </is>
@@ -10518,32 +11061,32 @@
           <t>'Applicants may be considered for graduate assistantships from the Department'</t>
         </is>
       </c>
-      <c r="F207" s="30" t="inlineStr">
+      <c r="F207" s="31" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,GA随申请自动考虑无需另申;个人陈述可写感兴趣的方向/教授</t>
         </is>
       </c>
-      <c r="G207" s="30" t="inlineStr">
+      <c r="G207" s="31" t="inlineStr">
         <is>
           <t>可以申请(系里可考虑授予GA,无需单独申请;当TA需满足伊州非母语TA英语要求)。先修:区域认证大学四年制学士;最后60学时GPA≥3.0;目的陈述+3位推荐人;无指定专业先修课</t>
         </is>
       </c>
-      <c r="H207" s="30" t="inlineStr">
+      <c r="H207" s="31" t="inlineStr">
         <is>
           <t>2027/2/1(按官网秋季截止2/1,2027待公布);GA随申请一并考虑,建议尽早提交</t>
         </is>
       </c>
-      <c r="I207" s="30" t="inlineStr">
+      <c r="I207" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不需要(官网未列GRE;Peterson's仍列GRE,疑已过时)</t>
         </is>
       </c>
-      <c r="J207" s="30" t="inlineStr">
+      <c r="J207" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不明确:ISU英语豁免指南列有美国区域认证学士学位这一豁免途径,但表格显示可能仅对应部分pathway,需向 InternationalAdmissions@IllinoisState.edu 确认;不豁免则 TOEFL ≥81,IELTS ≥6.5,Duolingo ≥110。当TA另需伊州非母语TA英语证明(如IELTS 8.0)</t>
         </is>
       </c>
-      <c r="K207" s="30" t="inlineStr">
+      <c r="K207" s="31" t="inlineStr">
         <is>
           <t>fcs@ilstu.edu(系办公室;研究生顾问 Dr. Jen Barnes,电话309-438-3558)</t>
         </is>
@@ -10580,27 +11123,27 @@
           <t>仅校级GA池:最低stipend $3,200/学期,部分至全额学费减免</t>
         </is>
       </c>
-      <c r="F208" s="30" t="inlineStr">
+      <c r="F208" s="31" t="inlineStr">
         <is>
           <t>不需要:经HAMPCAS统一申请,按项目整体录取,入围者需面试</t>
         </is>
       </c>
-      <c r="G208" s="30" t="inlineStr">
+      <c r="G208" s="31" t="inlineStr">
         <is>
           <t>可以申请(国际生可申请校级GA池)。先修:认证院校学士学位;累计GPA≥3.0(不足可用最近40学分的替代GPA);无指定专业先修课;经HAMPCAS申请,需面试</t>
         </is>
       </c>
-      <c r="H208" s="30" t="inlineStr">
+      <c r="H208" s="31" t="inlineStr">
         <is>
           <t>优先 3/1;需F-1签证的国际生 4/15;之后滚动审核至招满(按2025周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I208" s="30" t="inlineStr">
+      <c r="I208" s="31" t="inlineStr">
         <is>
           <t>不需要(官网明确不要求GRE/GMAT)</t>
         </is>
       </c>
-      <c r="J208" s="30" t="inlineStr">
+      <c r="J208" s="31" t="inlineStr">
         <is>
           <t>⚠️ 很可能否:ODU英语要求页列'在英语为官方语言国家的认证院校获学士/硕士学位'可满足要求(未点名美国,措辞有版本差异);否则 TOEFL iBT ≥79(2026/1/21后新制≥4.5),IELTS ≥6.5,Duolingo ≥120</t>
         </is>
@@ -10638,32 +11181,32 @@
           <t>'GRA positions advertised within the department when faculty have funded research'</t>
         </is>
       </c>
-      <c r="F209" s="30" t="inlineStr">
+      <c r="F209" s="31" t="inlineStr">
         <is>
           <t>不需要:项目整体综合录取,符合条件者需与教师进行简短面试</t>
         </is>
       </c>
-      <c r="G209" s="30" t="inlineStr">
+      <c r="G209" s="31" t="inlineStr">
         <is>
           <t>可以申请(GRA仅在教师有经费项目时系内招聘,不保证)。先修:区域认证大学学士;GPA≥3.0;医疗行业工作经验优先但非必需;需目标陈述、简历、成绩单(⚠️推荐信要求各页面说法不一);⚠️ F-1需确认就读校园面授班</t>
         </is>
       </c>
-      <c r="H209" s="30" t="inlineStr">
+      <c r="H209" s="31" t="inlineStr">
         <is>
           <t>优先截止:秋季 4/1(春季 11/1),之后视名额继续审核(按现行官网,2027待公布)</t>
         </is>
       </c>
-      <c r="I209" s="30" t="inlineStr">
+      <c r="I209" s="31" t="inlineStr">
         <is>
           <t>不需要(官网称GRE/GMAT已不再要求)</t>
         </is>
       </c>
-      <c r="J209" s="30" t="inlineStr">
+      <c r="J209" s="31" t="inlineStr">
         <is>
           <t>否(美国区域认证大学学位豁免,GMU全校政策)</t>
         </is>
       </c>
-      <c r="K209" s="30" t="inlineStr">
+      <c r="K209" s="31" t="inlineStr">
         <is>
           <t>muriyo@gmu.edu(MHA项目协调员 Dr. Maria Uriyo);masongrad@gmu.edu(研究生招生)</t>
         </is>
@@ -11306,7 +11849,7 @@
           <t>'A number of graduate assistantships awarded each year';GA含stipend+学费减免+医保;无硕士比例</t>
         </is>
       </c>
-      <c r="F225" s="30" t="inlineStr">
+      <c r="F225" s="31" t="inlineStr">
         <is>
           <t>不需要:MPH经SOPHAS按项目整体录取;GA多由教师科研经费资助,无正式申请流程,录取后可主动联系有经费的教师</t>
         </is>
@@ -11316,22 +11859,22 @@
           <t>未说明</t>
         </is>
       </c>
-      <c r="H225" s="30" t="inlineStr">
+      <c r="H225" s="31" t="inlineStr">
         <is>
           <t>⚠️ 资助/GA考虑截止 2027/1/5;最终截止 2027/5/1(据UGA Bulletin HPM方向页面,未标年份,按往年惯例推定,2027待公布)</t>
         </is>
       </c>
-      <c r="I225" s="30" t="inlineStr">
+      <c r="I225" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不需要(第三方称MPH已不要求GRE,UGA DrPH官网亦已取消;MPH页未直接确认)</t>
         </is>
       </c>
-      <c r="J225" s="30" t="inlineStr">
+      <c r="J225" s="31" t="inlineStr">
         <is>
           <t>否(美国学位豁免):UGA研究生院2025/3/12新政,美国认证院校学位免TOEFL/IELTS(个别院系可另行要求);否则TOEFL ≥80(口语/写作≥20)或IELTS ≥6.5(单项≥6.0),不接受Duolingo;如任TA另需满足TA英语政策</t>
         </is>
       </c>
-      <c r="K225" s="30" t="inlineStr">
+      <c r="K225" s="31" t="inlineStr">
         <is>
           <t>mph@uga.edu(校园MPH招生办);gradadm@uga.edu(研究生院招生)</t>
         </is>
@@ -11368,28 +11911,28 @@
           <t>校级:'Most assistantships are awarded to doctoral students';学院GA页未抓到</t>
         </is>
       </c>
-      <c r="F226" s="30" t="inlineStr">
+      <c r="F226" s="31" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,个人陈述可写感兴趣方向/教授;校级GA多给博士生</t>
         </is>
       </c>
-      <c r="G226" s="30" t="inlineStr">
+      <c r="G226" s="31" t="inlineStr">
         <is>
           <t>可以申请(国际生可申请;校级称GA多授予博士生,硕士资助有限)。先修:认证院校学士学位,本科GPA ≥3.0;需个人陈述、简历、成绩单、推荐信(官网说法2–3封不一);国际生另需财力证明等签证材料</t>
         </is>
       </c>
-      <c r="H226" s="30" t="inlineStr">
+      <c r="H226" s="31" t="inlineStr">
         <is>
           <t>⚠️ 官网说法不一:catalog称国际生秋季优先截止 3/15;国际招生页称秋季 6/15,截止后仍可能受理;建议 2027/3/15 前提交(按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I226" s="30" t="inlineStr">
+      <c r="I226" s="31" t="inlineStr">
         <is>
           <t>不需要(学院明确MPH/MS不要求GRE,仅PhD需要)</t>
         </is>
       </c>
       <c r="J226" s="22" t="n"/>
-      <c r="K226" s="30" t="inlineStr">
+      <c r="K226" s="31" t="inlineStr">
         <is>
           <t>publichealth@kent.edu(公共卫生学院总邮箱);⚠️ kbaker80@kent.edu(研究生项目助理协调员,目录信息待核实)</t>
         </is>
@@ -12182,32 +12725,32 @@
           <t>'limited number of tuition waivers to first-year';assistantships'rarely awarded in the first semester'</t>
         </is>
       </c>
-      <c r="F245" s="30" t="inlineStr">
+      <c r="F245" s="31" t="inlineStr">
         <is>
           <t>不需要:专业型硕士按项目整体录取,个人陈述可写感兴趣的教授</t>
         </is>
       </c>
-      <c r="G245" s="30" t="inlineStr">
+      <c r="G245" s="31" t="inlineStr">
         <is>
           <t>可以申请(国际生可获有限的首年学费减免;assistantship首学期很少发放)。先修:区域认证学士学位,研究生院最低GPA 3.0;无指定本科专业</t>
         </is>
       </c>
-      <c r="H245" s="30" t="inlineStr">
+      <c r="H245" s="31" t="inlineStr">
         <is>
           <t>资助优先 1/19;其后 2/22、3/22 两轮,3/22后滚动审核至开学前一个月;国际生最晚 5/25(按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I245" s="30" t="inlineStr">
+      <c r="I245" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不需要(第三方显示不要求GRE,官网未明确写出)</t>
         </is>
       </c>
-      <c r="J245" s="30" t="inlineStr">
+      <c r="J245" s="31" t="inlineStr">
         <is>
           <t>否(美国学位豁免):研究生院规定在美国区域认证院校获学士及以上学位者免交;否则 TOEFL ≥79(口语≥26)/IELTS ≥7</t>
         </is>
       </c>
-      <c r="K245" s="30" t="inlineStr">
+      <c r="K245" s="31" t="inlineStr">
         <is>
           <t>capla-grad@arizona.edu(CAPLA研究生项目协调员)</t>
         </is>
@@ -12244,32 +12787,32 @@
           <t>系有若干GTA(MS 1年,可续);GA按居民学费+stipend+≤9学分fee waiver</t>
         </is>
       </c>
-      <c r="F246" s="30" t="inlineStr">
+      <c r="F246" s="31" t="inlineStr">
         <is>
           <t>建议:小型项目,GTA由系分配,可先邮件项目主任 Thomas Albright 了解研究方向与助教机会</t>
         </is>
       </c>
-      <c r="G246" s="30" t="inlineStr">
+      <c r="G246" s="31" t="inlineStr">
         <is>
           <t>可以申请(系有少量GTA,国际生可申)。先修:学士学位,GPA ≥3.0;需修过入门统计课(可在第一学期补修);需目的陈述+3封推荐信</t>
         </is>
       </c>
-      <c r="H246" s="30" t="inlineStr">
+      <c r="H246" s="31" t="inlineStr">
         <is>
           <t>秋季 2/1(2/1前完成申请保证被考虑;按2026周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I246" s="30" t="inlineStr">
+      <c r="I246" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不明确:2022-23目录写需提交GRE成绩;研究生院称由项目自定,建议邮件确认</t>
         </is>
       </c>
-      <c r="J246" s="30" t="inlineStr">
+      <c r="J246" s="31" t="inlineStr">
         <is>
           <t>否(美国学位豁免):在美国认证英语授课院校在校(非网课)获学士及以上学位者免交;否则 TOEFL ≥79/IELTS ≥6.5</t>
         </is>
       </c>
-      <c r="K246" s="30" t="inlineStr">
+      <c r="K246" s="31" t="inlineStr">
         <is>
           <t>talbright@unr.edu(LUPP项目主任 Thomas Albright,⚠️来源较旧,需确认仍在任)</t>
         </is>
@@ -12306,18 +12849,18 @@
           <t>校级TA/RA/fellowship含stipend+tuition award;'in-state, out-of-state, or international student, you may be eligible'</t>
         </is>
       </c>
-      <c r="F247" s="30" t="inlineStr">
+      <c r="F247" s="31" t="inlineStr">
         <is>
           <t>不需要:专业型硕士按项目整体录取</t>
         </is>
       </c>
-      <c r="G247" s="30" t="inlineStr">
+      <c r="G247" s="31" t="inlineStr">
         <is>
           <t>可以申请(校级TA/RA/fellowship明确对国际生开放)。先修:区域认证学士学位;GPA ≥3.0正式录取,2.5–2.9可条件录取;需叙述性个人陈述+3封推荐信</t>
         </is>
       </c>
       <c r="H247" s="22" t="n"/>
-      <c r="I247" s="30" t="inlineStr">
+      <c r="I247" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不明确:Peterson's列GRE为部分申请者需提交,另有第三方称不需要,建议邮件确认</t>
         </is>
@@ -12356,32 +12899,32 @@
           <t>仅$1,000–8,000奖学金;无assistantship说明</t>
         </is>
       </c>
-      <c r="F248" s="30" t="inlineStr">
+      <c r="F248" s="31" t="inlineStr">
         <is>
           <t>不需要:专业型硕士按项目整体录取</t>
         </is>
       </c>
-      <c r="G248" s="30" t="inlineStr">
+      <c r="G248" s="31" t="inlineStr">
         <is>
           <t>可以申请,但资助仅$1,000–8,000奖学金,无assistantship说明。先修:须获学士学位,最低GPA 3.0;无指定本科专业</t>
         </is>
       </c>
-      <c r="H248" s="30" t="inlineStr">
+      <c r="H248" s="31" t="inlineStr">
         <is>
           <t>秋季:国际生 12/15,本国生 1/15(须按时才有奖学金资格);迟交至 5/1按名额审核且不可获奖学金(官网当前页日期,2027周期待确认)</t>
         </is>
       </c>
-      <c r="I248" s="30" t="inlineStr">
+      <c r="I248" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不需要(官网录取页未提GRE;第三方称GPA&lt;3.0时需提交)</t>
         </is>
       </c>
-      <c r="J248" s="30" t="inlineStr">
+      <c r="J248" s="31" t="inlineStr">
         <is>
           <t>否(美国学位豁免):在美国获学士及以上学位即满足英语要求;否则 TOEFL ≥79/IELTS ≥6.5</t>
         </is>
       </c>
-      <c r="K248" s="30" t="inlineStr">
+      <c r="K248" s="31" t="inlineStr">
         <is>
           <t>⚠️ 邮箱未在检索结果中显示:研究生招生经理 Jodi Stock(见学院staff页),学院电话 303-315-1000;jennifer.steffeljohnson@ucdenver.edu(MURP教师,⚠️来源可能过时)</t>
         </is>
@@ -13090,23 +13633,23 @@
           <t>'limited number of GTAs';州外学费减免仅第一年、只降到州内</t>
         </is>
       </c>
-      <c r="F265" s="30" t="inlineStr">
+      <c r="F265" s="31" t="inlineStr">
         <is>
           <t>⚠️ 官网未明确要求:按项目整体录取,可能面试;PSYS为读博/科研导向方向,建议陈述中写明匹配教授,可提前邮件联系</t>
         </is>
       </c>
-      <c r="G265" s="30" t="inlineStr">
+      <c r="G265" s="31" t="inlineStr">
         <is>
           <t>可以申请(GTA名额有限,州外学费减免仅第一年且只降到州内)。先修:期望心理学专业且心理学GPA≥3.0;非心理专业需≥21学分心理学课(含研究方法与统计,研究方法须为心理学课);总GPA≥3.0;3封推荐信(至少1封来自教授)、陈述、CV;只能申请一个方向</t>
         </is>
       </c>
       <c r="H265" s="22" t="n"/>
-      <c r="I265" s="30" t="inlineStr">
+      <c r="I265" s="31" t="inlineStr">
         <is>
           <t>不需要(官网FAQ:目前不考虑GRE)</t>
         </is>
       </c>
-      <c r="J265" s="30" t="inlineStr">
+      <c r="J265" s="31" t="inlineStr">
         <is>
           <t>否(美国学位豁免:UNCW研究生院认可美国认证院校学士学位免语言成绩;否则 TOEFL ≥79)</t>
         </is>
@@ -13144,28 +13687,28 @@
           <t>系分配TA/RA;校外GA'discounted tuition rates'</t>
         </is>
       </c>
-      <c r="F266" s="30" t="inlineStr">
+      <c r="F266" s="31" t="inlineStr">
         <is>
           <t>⚠️ 官网未明确:HF方向规模小、偏实验室制,建议提前联系HF方向教师(目录联系人 Michael Granaas)</t>
         </is>
       </c>
-      <c r="G266" s="30" t="inlineStr">
+      <c r="G266" s="31" t="inlineStr">
         <is>
           <t>可以申请。先修:认证院校学士学位;最低GPA 3.0;推荐信2封(新版目录,旧版3封)、statement of purpose、成绩单;申请费$35;MA含必修实习;分论文/非论文(30–36学分)</t>
         </is>
       </c>
-      <c r="H266" s="30" t="inlineStr">
+      <c r="H266" s="31" t="inlineStr">
         <is>
           <t>⚠️ HFES目录:优先 12/31;最终按名额滚动(开学前约4周);官网目录另列秋季 8/1;Peterson's 列 2/1;第三方称国际生 7/20。建议 2026/12/31 前提交并邮件确认</t>
         </is>
       </c>
-      <c r="I266" s="30" t="inlineStr">
+      <c r="I266" s="31" t="inlineStr">
         <is>
           <t>⚠️ 可能不需要:HFES目录称 Fall 2023 起免GRE,官网目录未见GRE要求,建议确认</t>
         </is>
       </c>
       <c r="J266" s="22" t="n"/>
-      <c r="K266" s="30" t="inlineStr">
+      <c r="K266" s="31" t="inlineStr">
         <is>
           <t>⚠️ Michael.Granaas@usd.edu(HFES目录所列项目联系人,可能过时);心理系电话 605-658-6140</t>
         </is>
@@ -13202,32 +13745,32 @@
           <t>校级GA'stipend and possible tuition remission';国际生页明列assistantship为资助途径</t>
         </is>
       </c>
-      <c r="F267" s="30" t="inlineStr">
+      <c r="F267" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不需要:按项目整体录取(MA要求论文),陈述中可写感兴趣的教授</t>
         </is>
       </c>
-      <c r="G267" s="30" t="inlineStr">
+      <c r="G267" s="31" t="inlineStr">
         <is>
           <t>可以申请(国际生页明列assistantship为资助途径)。⚠️ 先修(Peterson's):心理学≥15学分(含心理统计、研究方法);最低GPA 2.7(General)/3.2(Clinical方向);需推荐信、个人陈述</t>
         </is>
       </c>
-      <c r="H267" s="30" t="inlineStr">
+      <c r="H267" s="31" t="inlineStr">
         <is>
           <t>⚠️ 第三方:General Psychology 3/1(国际生同,资助申请同为3/1);Clinical方向 2/15 优先;另有来源称统一 2/15。建议 2027/2/15 前提交(按旧周期,2027待公布)</t>
         </is>
       </c>
-      <c r="I267" s="30" t="inlineStr">
+      <c r="I267" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不明确:Peterson's 列必需(Clinical要求V+Q≥300、单项≥148);另一来源称可选,建议确认</t>
         </is>
       </c>
-      <c r="J267" s="30" t="inlineStr">
+      <c r="J267" s="31" t="inlineStr">
         <is>
           <t>⚠️ 大概率否:第三方(Studee)称在美国区域认证院校获学士可豁免;官网写 TOEFL iBT ≥80(部分项目更高),未直接查到豁免条款,建议向 goglobalgraduate@udayton.edu 确认</t>
         </is>
       </c>
-      <c r="K267" s="30" t="inlineStr">
+      <c r="K267" s="31" t="inlineStr">
         <is>
           <t>gradadmission@udayton.edu(研究生招生办,通用);goglobalgraduate@udayton.edu(国际研究生招生)</t>
         </is>
@@ -13264,18 +13807,18 @@
           <t>仅校级GA(≤20h/周);奖学金$1–2k</t>
         </is>
       </c>
-      <c r="F268" s="30" t="inlineStr">
+      <c r="F268" s="31" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取;须完成6学分论文,陈述中可写感兴趣的教授</t>
         </is>
       </c>
-      <c r="G268" s="30" t="inlineStr">
+      <c r="G268" s="31" t="inlineStr">
         <is>
           <t>可以申请(仅校级GA,每周≤20小时)。先修(2025–26目录):本科最后60学分GPA≥3.0;统计和/或研究方法本科课成绩B以上;3封推荐信;500词目标陈述;CV。论文型项目,共36学分,为读博做准备</t>
         </is>
       </c>
       <c r="H268" s="22" t="n"/>
-      <c r="I268" s="30" t="inlineStr">
+      <c r="I268" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不需要:2025–26目录未列GRE(旧目录曾要求 V153/Q144),建议确认</t>
         </is>
@@ -13944,28 +14487,28 @@
           <t>'try our best to fund our terminal master's degree students when resources are available';TA/RA=stipend+9学分学费</t>
         </is>
       </c>
-      <c r="F284" s="30" t="inlineStr">
+      <c r="F284" s="31" t="inlineStr">
         <is>
           <t>不需要:按项目整体录取,SOP需写研究兴趣及希望合作的系内教师</t>
         </is>
       </c>
-      <c r="G284" s="30" t="inlineStr">
+      <c r="G284" s="31" t="inlineStr">
         <is>
           <t>可以申请,但系里资助(TA等)主要给MS-to-PhD和PhD-only申请者,terminal MS只在有资源时尽量资助。先修:官网未列最低GPA或具体先修学分;MS必修社会学理论、研究方法、社会统计(SOCI 5050/5200/5210或同等课程)。材料:CV、SOP、2封推荐信、$75申请费(GradCAS)</t>
         </is>
       </c>
-      <c r="H284" s="30" t="inlineStr">
+      <c r="H284" s="31" t="inlineStr">
         <is>
           <t>资助优先 2027/2/1(秋季);之后每月滚动审核至 2027/7/31;MS-only也可春季入学,春季截止 11/30(⚠️ 官网未注明年份,建议核实)</t>
         </is>
       </c>
-      <c r="I284" s="30" t="inlineStr">
+      <c r="I284" s="31" t="inlineStr">
         <is>
           <t>不需要(系官网:GRE不要求)</t>
         </is>
       </c>
       <c r="J284" s="22" t="n"/>
-      <c r="K284" s="30" t="inlineStr">
+      <c r="K284" s="31" t="inlineStr">
         <is>
           <t>William.Scarborough@unt.edu(研究生项目主任);sociology@unt.edu(系办公室)</t>
         </is>
@@ -14044,27 +14587,27 @@
           <t>'Assistantships are available to a few select graduate students';GA按州内学费计,州外差额靠另一奖学金;截止2/15</t>
         </is>
       </c>
-      <c r="F286" s="30" t="inlineStr">
+      <c r="F286" s="31" t="inlineStr">
         <is>
           <t>不适用:该项目已停止招生</t>
         </is>
       </c>
-      <c r="G286" s="30" t="inlineStr">
+      <c r="G286" s="31" t="inlineStr">
         <is>
           <t>❌ 该项目已停止招收新生(ODU官网:this program is no longer accepting new students,学位须于2025年8月前完成;目录写已建议关闭)。原要求:GPA≥3.0,本科社会学或刑事司法≥12学分,含理论、研究方法、统计。系里目前只开设犯罪学与刑事司法PhD</t>
         </is>
       </c>
-      <c r="H286" s="30" t="inlineStr">
+      <c r="H286" s="31" t="inlineStr">
         <is>
           <t>❌ 已停招;原截止:GA 2/15,最终 3/1(仅秋季入学)</t>
         </is>
       </c>
-      <c r="I286" s="30" t="inlineStr">
+      <c r="I286" s="31" t="inlineStr">
         <is>
           <t>必需(原要求;项目已停招)</t>
         </is>
       </c>
-      <c r="J286" s="30" t="inlineStr">
+      <c r="J286" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不明确:原要求非母语国际生 TOEFL 550(纸考)等,未写美国学位豁免;项目已停招</t>
         </is>
@@ -14144,28 +14687,28 @@
           <t>硕士'仅部分资助';merit 奖学金 ≤50% 州内学费;International Chancellor's Scholarship</t>
         </is>
       </c>
-      <c r="F288" s="30" t="inlineStr">
+      <c r="F288" s="31" t="inlineStr">
         <is>
           <t>不需要:硕士按项目整体录取(只有PhD申请者需在个人陈述中写希望合作的教师)</t>
         </is>
       </c>
-      <c r="G288" s="30" t="inlineStr">
+      <c r="G288" s="31" t="inlineStr">
         <is>
           <t>可以申请(有国际生专项奖 International Chancellor's Scholarship)。⚠️ 先修(按2023-2025目录):社会科学或相关专业本科,GPA≥3.3(录取者通常≥3.5);统计和研究方法课程成绩优秀;材料:成绩单、CV、3封推荐信</t>
         </is>
       </c>
       <c r="H288" s="22" t="n"/>
-      <c r="I288" s="30" t="inlineStr">
+      <c r="I288" s="31" t="inlineStr">
         <is>
           <t>⚠️ 目录未提GRE,可能不需要,建议确认</t>
         </is>
       </c>
-      <c r="J288" s="30" t="inlineStr">
+      <c r="J288" s="31" t="inlineStr">
         <is>
           <t>⚠️ 不明确:目录写英语为第二语言的外国学生都需TOEFL,未写美国学位豁免,建议邮件确认</t>
         </is>
       </c>
-      <c r="K288" s="30" t="inlineStr">
+      <c r="K288" s="31" t="inlineStr">
         <is>
           <t>kristin.august@rutgers.edu(项目主任 Kristin August)</t>
         </is>

</xml_diff>